<commit_message>
Add NVIDIA P4 acquisition to Lab inventory and recent arrivals
</commit_message>
<xml_diff>
--- a/public/lab/hack-lab-inventory.xlsx
+++ b/public/lab/hack-lab-inventory.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R29282b884beb4024"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory" sheetId="2" r:id="Rf754523ccc7248b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Power model" sheetId="3" r:id="R6af80ea00e9c4a20"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R8319e62e90eb446f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory" sheetId="2" r:id="R7fb7f7fec9304c99"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Power model" sheetId="3" r:id="Rc302cc486238468f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -278,8 +278,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="LabInventory" displayName="LabInventory" ref="A7:J59" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A7:J59"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="LabInventory" displayName="LabInventory" ref="A7:J60" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A7:J60"/>
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="Item ID"/>
     <x:tableColumn id="2" name="Equipment and specifications"/>
@@ -543,7 +543,7 @@
         <x:v>Snapshot</x:v>
       </x:c>
       <x:c r="B4" s="6" t="n">
-        <x:v>46277.5</x:v>
+        <x:v>46278.5</x:v>
       </x:c>
       <x:c r="C4" s="3"/>
       <x:c r="D4" s="3"/>
@@ -568,9 +568,9 @@
       <x:c r="A7" s="3" t="str">
         <x:v>Compute and add-ons</x:v>
       </x:c>
-      <x:c r="B7" s="15" t="n">
-        <x:f>IF(COUNT('Inventory'!G8:G59)=ROWS('Inventory'!G8:G59),SUMIFS('Inventory'!G8:G59,'Inventory'!J8:J59,A7),"Missing input")</x:f>
-        <x:v>28244</x:v>
+      <x:c r="B7" s="15" t="str">
+        <x:f>IF(COUNTIFS('Inventory'!J8:J60,A7,'Inventory'!G8:G60,"Missing input")=0,SUMIFS('Inventory'!G8:G60,'Inventory'!J8:J60,A7),"Missing input")</x:f>
+        <x:v>Missing input</x:v>
       </x:c>
       <x:c r="C7" s="3"/>
       <x:c r="D7" s="3"/>
@@ -580,7 +580,7 @@
         <x:v>Rack and shared</x:v>
       </x:c>
       <x:c r="B8" s="15" t="n">
-        <x:f>IF(COUNT('Inventory'!G8:G59)=ROWS('Inventory'!G8:G59),SUMIFS('Inventory'!G8:G59,'Inventory'!J8:J59,A8),"Missing input")</x:f>
+        <x:f>IF(COUNTIFS('Inventory'!J8:J60,A8,'Inventory'!G8:G60,"Missing input")=0,SUMIFS('Inventory'!G8:G60,'Inventory'!J8:J60,A8),"Missing input")</x:f>
         <x:v>1505</x:v>
       </x:c>
       <x:c r="C8" s="3"/>
@@ -590,22 +590,27 @@
       <x:c r="A9" s="18" t="str">
         <x:v>Total replacement estimate</x:v>
       </x:c>
-      <x:c r="B9" s="19" t="n">
+      <x:c r="B9" s="19" t="str">
         <x:f>IF(COUNT(B7:B8)=2,SUM(B7:B8),"Missing input")</x:f>
-        <x:v>29749</x:v>
+        <x:v>Missing input</x:v>
       </x:c>
       <x:c r="C9" s="3"/>
       <x:c r="D9" s="3"/>
     </x:row>
     <x:row r="10" ht="24" customHeight="1">
-      <x:c r="A10" s="3"/>
-      <x:c r="B10" s="3"/>
+      <x:c r="A10" s="3" t="str">
+        <x:v>Priced equipment subtotal</x:v>
+      </x:c>
+      <x:c r="B10" s="15" t="n">
+        <x:f>SUM('Inventory'!G8:G60)</x:f>
+        <x:v>29749</x:v>
+      </x:c>
       <x:c r="C10" s="3"/>
       <x:c r="D10" s="3"/>
     </x:row>
     <x:row r="11" ht="24" customHeight="1">
       <x:c r="A11" s="20" t="str">
-        <x:v>Dated reference prices and allowances. This is not an amount paid or a current quote.</x:v>
+        <x:v>Full total needs all prices. Subtotal excludes unpriced equipment; it is not an amount paid.</x:v>
       </x:c>
       <x:c r="B11" s="3"/>
       <x:c r="C11" s="3"/>
@@ -727,7 +732,7 @@
     </x:row>
     <x:row r="24" ht="24" customHeight="1">
       <x:c r="A24" s="20" t="str">
-        <x:v>Agent Blade watts are projected for a populated board. Actual draw is not yet published.</x:v>
+        <x:v>Agent Blade watts are projected. Newly acquired equipment is excluded until modeled.</x:v>
       </x:c>
       <x:c r="B24" s="3"/>
       <x:c r="C24" s="3"/>
@@ -898,7 +903,7 @@
     </x:row>
     <x:row r="5" ht="24" customHeight="1">
       <x:c r="A5" s="20" t="str">
-        <x:v>Power estimates are on the Power model tab. Shared components and spare cards do not add watts.</x:v>
+        <x:v>Blank costs are unknown, not zero. Newly acquired equipment has its status in the source note.</x:v>
       </x:c>
       <x:c r="B5" s="3"/>
       <x:c r="C5" s="3"/>
@@ -2935,50 +2940,71 @@
 https://www.bestbuy.com/site/searchpage.jsp?id=pcat17071&amp;st=mini+hdmi+adapter+to+hdmi</x:v>
       </x:c>
     </x:row>
-    <x:row r="60" ht="24" customHeight="1">
-      <x:c r="A60" s="3"/>
-      <x:c r="B60" s="3"/>
-      <x:c r="C60" s="3"/>
-      <x:c r="D60" s="3"/>
-      <x:c r="E60" s="3"/>
-      <x:c r="F60" s="3"/>
-      <x:c r="G60" s="3"/>
-      <x:c r="H60" s="3"/>
-      <x:c r="I60" s="3"/>
-      <x:c r="J60" s="3"/>
+    <x:row r="60" ht="57" customHeight="1">
+      <x:c r="A60" s="3" t="str">
+        <x:v>EQ-53</x:v>
+      </x:c>
+      <x:c r="B60" s="30" t="str">
+        <x:v>NVIDIA P4 GPU, 8 GB memory</x:v>
+      </x:c>
+      <x:c r="C60" s="38" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D60" s="39"/>
+      <x:c r="E60" s="39" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F60" s="40" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G60" s="41" t="str">
+        <x:f>IF(COUNT(C60:F60)=4,ROUND(C60*(D60+E60),0)+F60,"Missing input")</x:f>
+        <x:v>Missing input</x:v>
+      </x:c>
+      <x:c r="H60" s="42" t="str">
+        <x:v>none</x:v>
+      </x:c>
+      <x:c r="I60" s="30" t="str">
+        <x:v>Not modeled: installation and power use unconfirmed</x:v>
+      </x:c>
+      <x:c r="J60" s="30" t="str">
+        <x:v>Compute and add-ons</x:v>
+      </x:c>
       <x:c r="K60" s="3"/>
-      <x:c r="L60" s="3"/>
-    </x:row>
-    <x:row r="61" ht="30" customHeight="1">
-      <x:c r="A61" s="18" t="str">
-        <x:v>Total replacement estimate</x:v>
-      </x:c>
-      <x:c r="B61" s="18"/>
-      <x:c r="C61" s="18"/>
-      <x:c r="D61" s="18"/>
-      <x:c r="E61" s="18"/>
-      <x:c r="F61" s="18"/>
-      <x:c r="G61" s="19" t="n">
-        <x:f>IF(COUNT(G8:G59)=ROWS(G8:G59),SUM(G8:G59),"Missing input")</x:f>
-        <x:v>29749</x:v>
-      </x:c>
-      <x:c r="H61" s="18"/>
-      <x:c r="I61" s="18"/>
-      <x:c r="J61" s="18"/>
+      <x:c r="L60" s="32" t="str">
+        <x:v>Acquisition reported by Shannon Duncan on September 13, 2026. Installation and availability unconfirmed. No price supplied.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="24" customHeight="1">
+      <x:c r="A61" s="3"/>
+      <x:c r="B61" s="3"/>
+      <x:c r="C61" s="3"/>
+      <x:c r="D61" s="3"/>
+      <x:c r="E61" s="3"/>
+      <x:c r="F61" s="3"/>
+      <x:c r="G61" s="3"/>
+      <x:c r="H61" s="3"/>
+      <x:c r="I61" s="3"/>
+      <x:c r="J61" s="3"/>
       <x:c r="K61" s="3"/>
       <x:c r="L61" s="3"/>
     </x:row>
-    <x:row r="62" ht="24" customHeight="1">
-      <x:c r="A62" s="3"/>
-      <x:c r="B62" s="3"/>
-      <x:c r="C62" s="3"/>
-      <x:c r="D62" s="3"/>
-      <x:c r="E62" s="3"/>
-      <x:c r="F62" s="3"/>
-      <x:c r="G62" s="3"/>
-      <x:c r="H62" s="3"/>
-      <x:c r="I62" s="3"/>
-      <x:c r="J62" s="3"/>
+    <x:row r="62" ht="30" customHeight="1">
+      <x:c r="A62" s="18" t="str">
+        <x:v>Total replacement estimate</x:v>
+      </x:c>
+      <x:c r="B62" s="18"/>
+      <x:c r="C62" s="18"/>
+      <x:c r="D62" s="18"/>
+      <x:c r="E62" s="18"/>
+      <x:c r="F62" s="18"/>
+      <x:c r="G62" s="19" t="str">
+        <x:f>IF(COUNT(G8:G60)=ROWS(G8:G60),SUM(G8:G60),"Missing input")</x:f>
+        <x:v>Missing input</x:v>
+      </x:c>
+      <x:c r="H62" s="18"/>
+      <x:c r="I62" s="18"/>
+      <x:c r="J62" s="18"/>
       <x:c r="K62" s="3"/>
       <x:c r="L62" s="3"/>
     </x:row>
@@ -3010,21 +3036,35 @@
       <x:c r="K64" s="3"/>
       <x:c r="L64" s="3"/>
     </x:row>
+    <x:row r="65" ht="24" customHeight="1">
+      <x:c r="A65" s="3"/>
+      <x:c r="B65" s="3"/>
+      <x:c r="C65" s="3"/>
+      <x:c r="D65" s="3"/>
+      <x:c r="E65" s="3"/>
+      <x:c r="F65" s="3"/>
+      <x:c r="G65" s="3"/>
+      <x:c r="H65" s="3"/>
+      <x:c r="I65" s="3"/>
+      <x:c r="J65" s="3"/>
+      <x:c r="K65" s="3"/>
+      <x:c r="L65" s="3"/>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="G8:G59">
+  <x:conditionalFormatting sqref="G8:G60">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Missing input"/>
   </x:conditionalFormatting>
   <x:dataValidations count="2">
-    <x:dataValidation type="whole" operator="greaterThanOrEqual" sqref="C8:C59">
+    <x:dataValidation type="whole" operator="greaterThanOrEqual" sqref="C8:C60">
       <x:formula1>0</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="decimal" operator="greaterThanOrEqual" sqref="D8:E59">
+    <x:dataValidation type="decimal" operator="greaterThanOrEqual" sqref="D8:E60">
       <x:formula1>0</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ad4f69418a54a48"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc0e611ef6e4472e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3868,7 +3908,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f86e87428514861"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R65e4928c354d49c9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Split active and completed projects and record new lab hardware
</commit_message>
<xml_diff>
--- a/public/lab/hack-lab-inventory.xlsx
+++ b/public/lab/hack-lab-inventory.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R8319e62e90eb446f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory" sheetId="2" r:id="R7fb7f7fec9304c99"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Power model" sheetId="3" r:id="Rc302cc486238468f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R3a8ee0d0fc8b4ec0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory" sheetId="2" r:id="Rdcf9ebeaef8e4223"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Power model" sheetId="3" r:id="Ra718c3ec8d094731"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -278,8 +278,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="LabInventory" displayName="LabInventory" ref="A7:J60" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A7:J60"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="LabInventory" displayName="LabInventory" ref="A7:J67" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A7:J67"/>
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="Item ID"/>
     <x:tableColumn id="2" name="Equipment and specifications"/>
@@ -543,7 +543,7 @@
         <x:v>Snapshot</x:v>
       </x:c>
       <x:c r="B4" s="6" t="n">
-        <x:v>46278.5</x:v>
+        <x:v>46283.5</x:v>
       </x:c>
       <x:c r="C4" s="3"/>
       <x:c r="D4" s="3"/>
@@ -569,7 +569,7 @@
         <x:v>Compute and add-ons</x:v>
       </x:c>
       <x:c r="B7" s="15" t="str">
-        <x:f>IF(COUNTIFS('Inventory'!J8:J60,A7,'Inventory'!G8:G60,"Missing input")=0,SUMIFS('Inventory'!G8:G60,'Inventory'!J8:J60,A7),"Missing input")</x:f>
+        <x:f>IF(COUNTIFS('Inventory'!J8:J67,A7,'Inventory'!G8:G67,"Missing input")=0,SUMIFS('Inventory'!G8:G67,'Inventory'!J8:J67,A7),"Missing input")</x:f>
         <x:v>Missing input</x:v>
       </x:c>
       <x:c r="C7" s="3"/>
@@ -579,9 +579,9 @@
       <x:c r="A8" s="3" t="str">
         <x:v>Rack and shared</x:v>
       </x:c>
-      <x:c r="B8" s="15" t="n">
-        <x:f>IF(COUNTIFS('Inventory'!J8:J60,A8,'Inventory'!G8:G60,"Missing input")=0,SUMIFS('Inventory'!G8:G60,'Inventory'!J8:J60,A8),"Missing input")</x:f>
-        <x:v>1505</x:v>
+      <x:c r="B8" s="15" t="str">
+        <x:f>IF(COUNTIFS('Inventory'!J8:J67,A8,'Inventory'!G8:G67,"Missing input")=0,SUMIFS('Inventory'!G8:G67,'Inventory'!J8:J67,A8),"Missing input")</x:f>
+        <x:v>Missing input</x:v>
       </x:c>
       <x:c r="C8" s="3"/>
       <x:c r="D8" s="3"/>
@@ -602,8 +602,8 @@
         <x:v>Priced equipment subtotal</x:v>
       </x:c>
       <x:c r="B10" s="15" t="n">
-        <x:f>SUM('Inventory'!G8:G60)</x:f>
-        <x:v>29749</x:v>
+        <x:f>SUM('Inventory'!G8:G67)</x:f>
+        <x:v>30813</x:v>
       </x:c>
       <x:c r="C10" s="3"/>
       <x:c r="D10" s="3"/>
@@ -794,7 +794,7 @@
     </x:row>
     <x:row r="32" ht="24" customHeight="1">
       <x:c r="A32" s="20" t="str">
-        <x:v>Prices are from September 11, 2026, with the network switch updated September 12.</x:v>
+        <x:v>Reference prices: September 11–12, 2026; reported acquisition costs: September 18.</x:v>
       </x:c>
       <x:c r="B32" s="3"/>
       <x:c r="C32" s="3"/>
@@ -2975,96 +2975,345 @@
         <x:v>Acquisition reported by Shannon Duncan on September 13, 2026. Installation and availability unconfirmed. No price supplied.</x:v>
       </x:c>
     </x:row>
-    <x:row r="61" ht="24" customHeight="1">
-      <x:c r="A61" s="3"/>
-      <x:c r="B61" s="3"/>
-      <x:c r="C61" s="3"/>
-      <x:c r="D61" s="3"/>
-      <x:c r="E61" s="3"/>
-      <x:c r="F61" s="3"/>
-      <x:c r="G61" s="3"/>
-      <x:c r="H61" s="3"/>
-      <x:c r="I61" s="3"/>
-      <x:c r="J61" s="3"/>
+    <x:row r="61" ht="57" customHeight="1">
+      <x:c r="A61" s="16" t="str">
+        <x:v>EQ-54</x:v>
+      </x:c>
+      <x:c r="B61" s="43" t="str">
+        <x:v>CyberPower PR2200LCDSL Smart App Sinewave UPS, 2070 VA / 1980 W, 7 outlets, AVR, mini-tower</x:v>
+      </x:c>
+      <x:c r="C61" s="38" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D61" s="39" t="n">
+        <x:v>995</x:v>
+      </x:c>
+      <x:c r="E61" s="39" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F61" s="40" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G61" s="41" t="n">
+        <x:f>IF(COUNT(C61:F61)=4,ROUND(C61*(D61+E61),0)+F61,"Missing input")</x:f>
+        <x:v>995</x:v>
+      </x:c>
+      <x:c r="H61" s="42" t="str">
+        <x:v>none</x:v>
+      </x:c>
+      <x:c r="I61" s="30" t="str">
+        <x:v>Not modeled: replacement of or addition to the existing UPS branch is unconfirmed</x:v>
+      </x:c>
+      <x:c r="J61" s="30" t="str">
+        <x:v>Rack and shared</x:v>
+      </x:c>
       <x:c r="K61" s="3"/>
-      <x:c r="L61" s="3"/>
-    </x:row>
-    <x:row r="62" ht="30" customHeight="1">
-      <x:c r="A62" s="18" t="str">
+      <x:c r="L61" s="32" t="str">
+        <x:v>Acquisition and $995 cost reported by Shannon Duncan on September 18, 2026. Its rated output is not a wall-power measurement; installation and overhead are not yet modeled.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="57" customHeight="1">
+      <x:c r="A62" s="3" t="str">
+        <x:v>EQ-55</x:v>
+      </x:c>
+      <x:c r="B62" s="30" t="str">
+        <x:v>WEP 605D-III DC variable bench power supply, 60 V / 5 A</x:v>
+      </x:c>
+      <x:c r="C62" s="38" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D62" s="39" t="n">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="E62" s="39" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F62" s="40" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G62" s="41" t="n">
+        <x:f>IF(COUNT(C62:F62)=4,ROUND(C62*(D62+E62),0)+F62,"Missing input")</x:f>
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="H62" s="42" t="str">
+        <x:v>none</x:v>
+      </x:c>
+      <x:c r="I62" s="30" t="str">
+        <x:v>Not modeled: bench use and duty cycle unconfirmed</x:v>
+      </x:c>
+      <x:c r="J62" s="30" t="str">
+        <x:v>Compute and add-ons</x:v>
+      </x:c>
+      <x:c r="K62" s="3"/>
+      <x:c r="L62" s="32" t="str">
+        <x:v>Acquisition and $69 cost reported by Shannon Duncan on September 18, 2026. Output rating is not a wall-power measurement.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="57" customHeight="1">
+      <x:c r="A63" s="16" t="str">
+        <x:v>EQ-56</x:v>
+      </x:c>
+      <x:c r="B63" s="43" t="str">
+        <x:v>Luckfox Pico Mini A</x:v>
+      </x:c>
+      <x:c r="C63" s="38" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D63" s="39"/>
+      <x:c r="E63" s="39" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F63" s="40" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G63" s="41" t="str">
+        <x:f>IF(COUNT(C63:F63)=4,ROUND(C63*(D63+E63),0)+F63,"Missing input")</x:f>
+        <x:v>Missing input</x:v>
+      </x:c>
+      <x:c r="H63" s="42" t="str">
+        <x:v>none</x:v>
+      </x:c>
+      <x:c r="I63" s="30" t="str">
+        <x:v>Not modeled: configuration and active use unconfirmed</x:v>
+      </x:c>
+      <x:c r="J63" s="30" t="str">
+        <x:v>Compute and add-ons</x:v>
+      </x:c>
+      <x:c r="K63" s="3"/>
+      <x:c r="L63" s="32" t="str">
+        <x:v>Acquisition reported by Shannon Duncan on September 18, 2026. Price, configuration, and active use unconfirmed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="57" customHeight="1">
+      <x:c r="A64" s="3" t="str">
+        <x:v>EQ-57</x:v>
+      </x:c>
+      <x:c r="B64" s="30" t="str">
+        <x:v>Sipeed NanoKVM</x:v>
+      </x:c>
+      <x:c r="C64" s="38" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D64" s="39"/>
+      <x:c r="E64" s="39" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F64" s="40" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G64" s="41" t="str">
+        <x:f>IF(COUNT(C64:F64)=4,ROUND(C64*(D64+E64),0)+F64,"Missing input")</x:f>
+        <x:v>Missing input</x:v>
+      </x:c>
+      <x:c r="H64" s="42" t="str">
+        <x:v>none</x:v>
+      </x:c>
+      <x:c r="I64" s="30" t="str">
+        <x:v>Not modeled: installation and power use unconfirmed</x:v>
+      </x:c>
+      <x:c r="J64" s="30" t="str">
+        <x:v>Rack and shared</x:v>
+      </x:c>
+      <x:c r="K64" s="3"/>
+      <x:c r="L64" s="32" t="str">
+        <x:v>Acquisition reported by Shannon Duncan on September 18, 2026. Price and installation unconfirmed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" ht="57" customHeight="1">
+      <x:c r="A65" s="16" t="str">
+        <x:v>EQ-58</x:v>
+      </x:c>
+      <x:c r="B65" s="43" t="str">
+        <x:v>Grove Vision AI Module V2</x:v>
+      </x:c>
+      <x:c r="C65" s="38" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D65" s="39"/>
+      <x:c r="E65" s="39" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F65" s="40" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G65" s="41" t="str">
+        <x:f>IF(COUNT(C65:F65)=4,ROUND(C65*(D65+E65),0)+F65,"Missing input")</x:f>
+        <x:v>Missing input</x:v>
+      </x:c>
+      <x:c r="H65" s="42" t="str">
+        <x:v>none</x:v>
+      </x:c>
+      <x:c r="I65" s="30" t="str">
+        <x:v>Not modeled: project assignment and active use unconfirmed</x:v>
+      </x:c>
+      <x:c r="J65" s="30" t="str">
+        <x:v>Compute and add-ons</x:v>
+      </x:c>
+      <x:c r="K65" s="3"/>
+      <x:c r="L65" s="32" t="str">
+        <x:v>Acquisition reported by Shannon Duncan on September 18, 2026. Price and project assignment unconfirmed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="57" customHeight="1">
+      <x:c r="A66" s="3" t="str">
+        <x:v>EQ-59</x:v>
+      </x:c>
+      <x:c r="B66" s="30" t="str">
+        <x:v>Soldering iron setup</x:v>
+      </x:c>
+      <x:c r="C66" s="38" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D66" s="39"/>
+      <x:c r="E66" s="39" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F66" s="40" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G66" s="41" t="str">
+        <x:f>IF(COUNT(C66:F66)=4,ROUND(C66*(D66+E66),0)+F66,"Missing input")</x:f>
+        <x:v>Missing input</x:v>
+      </x:c>
+      <x:c r="H66" s="42" t="str">
+        <x:v>none</x:v>
+      </x:c>
+      <x:c r="I66" s="30" t="str">
+        <x:v>Not modeled: model and duty cycle unconfirmed</x:v>
+      </x:c>
+      <x:c r="J66" s="30" t="str">
+        <x:v>Compute and add-ons</x:v>
+      </x:c>
+      <x:c r="K66" s="3"/>
+      <x:c r="L66" s="32" t="str">
+        <x:v>Acquisition reported by Shannon Duncan on September 18, 2026. Model, price, and active power use unconfirmed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="57" customHeight="1">
+      <x:c r="A67" s="16" t="str">
+        <x:v>EQ-60</x:v>
+      </x:c>
+      <x:c r="B67" s="43" t="str">
+        <x:v>M5Stack CoreS3 ESP32-S3 development kit</x:v>
+      </x:c>
+      <x:c r="C67" s="38" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D67" s="39"/>
+      <x:c r="E67" s="39" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F67" s="40" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G67" s="41" t="str">
+        <x:f>IF(COUNT(C67:F67)=4,ROUND(C67*(D67+E67),0)+F67,"Missing input")</x:f>
+        <x:v>Missing input</x:v>
+      </x:c>
+      <x:c r="H67" s="42" t="str">
+        <x:v>none</x:v>
+      </x:c>
+      <x:c r="I67" s="30" t="str">
+        <x:v>Not modeled: project assignment and active use unconfirmed</x:v>
+      </x:c>
+      <x:c r="J67" s="30" t="str">
+        <x:v>Compute and add-ons</x:v>
+      </x:c>
+      <x:c r="K67" s="3"/>
+      <x:c r="L67" s="32" t="str">
+        <x:v>Acquisition reported by Shannon Duncan on September 18, 2026. Price and project assignment unconfirmed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68" ht="24" customHeight="1">
+      <x:c r="A68" s="3"/>
+      <x:c r="B68" s="3"/>
+      <x:c r="C68" s="3"/>
+      <x:c r="D68" s="3"/>
+      <x:c r="E68" s="3"/>
+      <x:c r="F68" s="3"/>
+      <x:c r="G68" s="3"/>
+      <x:c r="H68" s="3"/>
+      <x:c r="I68" s="3"/>
+      <x:c r="J68" s="3"/>
+      <x:c r="K68" s="3"/>
+      <x:c r="L68" s="3"/>
+    </x:row>
+    <x:row r="69" ht="30" customHeight="1">
+      <x:c r="A69" s="18" t="str">
         <x:v>Total replacement estimate</x:v>
       </x:c>
-      <x:c r="B62" s="18"/>
-      <x:c r="C62" s="18"/>
-      <x:c r="D62" s="18"/>
-      <x:c r="E62" s="18"/>
-      <x:c r="F62" s="18"/>
-      <x:c r="G62" s="19" t="str">
-        <x:f>IF(COUNT(G8:G60)=ROWS(G8:G60),SUM(G8:G60),"Missing input")</x:f>
+      <x:c r="B69" s="18"/>
+      <x:c r="C69" s="18"/>
+      <x:c r="D69" s="18"/>
+      <x:c r="E69" s="18"/>
+      <x:c r="F69" s="18"/>
+      <x:c r="G69" s="19" t="str">
+        <x:f>IF(COUNT(G8:G67)=ROWS(G8:G67),SUM(G8:G67),"Missing input")</x:f>
         <x:v>Missing input</x:v>
       </x:c>
-      <x:c r="H62" s="18"/>
-      <x:c r="I62" s="18"/>
-      <x:c r="J62" s="18"/>
-      <x:c r="K62" s="3"/>
-      <x:c r="L62" s="3"/>
-    </x:row>
-    <x:row r="63" ht="24" customHeight="1">
-      <x:c r="A63" s="3"/>
-      <x:c r="B63" s="3"/>
-      <x:c r="C63" s="3"/>
-      <x:c r="D63" s="3"/>
-      <x:c r="E63" s="3"/>
-      <x:c r="F63" s="3"/>
-      <x:c r="G63" s="3"/>
-      <x:c r="H63" s="3"/>
-      <x:c r="I63" s="3"/>
-      <x:c r="J63" s="3"/>
-      <x:c r="K63" s="3"/>
-      <x:c r="L63" s="3"/>
-    </x:row>
-    <x:row r="64" ht="24" customHeight="1">
-      <x:c r="A64" s="3"/>
-      <x:c r="B64" s="3"/>
-      <x:c r="C64" s="3"/>
-      <x:c r="D64" s="3"/>
-      <x:c r="E64" s="3"/>
-      <x:c r="F64" s="3"/>
-      <x:c r="G64" s="3"/>
-      <x:c r="H64" s="3"/>
-      <x:c r="I64" s="3"/>
-      <x:c r="J64" s="3"/>
-      <x:c r="K64" s="3"/>
-      <x:c r="L64" s="3"/>
-    </x:row>
-    <x:row r="65" ht="24" customHeight="1">
-      <x:c r="A65" s="3"/>
-      <x:c r="B65" s="3"/>
-      <x:c r="C65" s="3"/>
-      <x:c r="D65" s="3"/>
-      <x:c r="E65" s="3"/>
-      <x:c r="F65" s="3"/>
-      <x:c r="G65" s="3"/>
-      <x:c r="H65" s="3"/>
-      <x:c r="I65" s="3"/>
-      <x:c r="J65" s="3"/>
-      <x:c r="K65" s="3"/>
-      <x:c r="L65" s="3"/>
+      <x:c r="H69" s="18"/>
+      <x:c r="I69" s="18"/>
+      <x:c r="J69" s="18"/>
+      <x:c r="K69" s="3"/>
+      <x:c r="L69" s="3"/>
+    </x:row>
+    <x:row r="70" ht="24" customHeight="1">
+      <x:c r="A70" s="3"/>
+      <x:c r="B70" s="3"/>
+      <x:c r="C70" s="3"/>
+      <x:c r="D70" s="3"/>
+      <x:c r="E70" s="3"/>
+      <x:c r="F70" s="3"/>
+      <x:c r="G70" s="3"/>
+      <x:c r="H70" s="3"/>
+      <x:c r="I70" s="3"/>
+      <x:c r="J70" s="3"/>
+      <x:c r="K70" s="3"/>
+      <x:c r="L70" s="3"/>
+    </x:row>
+    <x:row r="71" ht="24" customHeight="1">
+      <x:c r="A71" s="3"/>
+      <x:c r="B71" s="3"/>
+      <x:c r="C71" s="3"/>
+      <x:c r="D71" s="3"/>
+      <x:c r="E71" s="3"/>
+      <x:c r="F71" s="3"/>
+      <x:c r="G71" s="3"/>
+      <x:c r="H71" s="3"/>
+      <x:c r="I71" s="3"/>
+      <x:c r="J71" s="3"/>
+      <x:c r="K71" s="3"/>
+      <x:c r="L71" s="3"/>
+    </x:row>
+    <x:row r="72" ht="24" customHeight="1">
+      <x:c r="A72" s="3"/>
+      <x:c r="B72" s="3"/>
+      <x:c r="C72" s="3"/>
+      <x:c r="D72" s="3"/>
+      <x:c r="E72" s="3"/>
+      <x:c r="F72" s="3"/>
+      <x:c r="G72" s="3"/>
+      <x:c r="H72" s="3"/>
+      <x:c r="I72" s="3"/>
+      <x:c r="J72" s="3"/>
+      <x:c r="K72" s="3"/>
+      <x:c r="L72" s="3"/>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="G8:G60">
+  <x:conditionalFormatting sqref="G8:G67">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Missing input"/>
   </x:conditionalFormatting>
   <x:dataValidations count="2">
-    <x:dataValidation type="whole" operator="greaterThanOrEqual" sqref="C8:C60">
+    <x:dataValidation type="whole" operator="greaterThanOrEqual" sqref="C8:C67">
       <x:formula1>0</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="decimal" operator="greaterThanOrEqual" sqref="D8:E60">
+    <x:dataValidation type="decimal" operator="greaterThanOrEqual" sqref="D8:E67">
       <x:formula1>0</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc0e611ef6e4472e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R650c21c70b554253"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3908,7 +4157,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R65e4928c354d49c9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbf31bd9d29d5407b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Research recent hardware costs and power references
</commit_message>
<xml_diff>
--- a/public/lab/hack-lab-inventory.xlsx
+++ b/public/lab/hack-lab-inventory.xlsx
@@ -2,9 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R3a8ee0d0fc8b4ec0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory" sheetId="2" r:id="Rdcf9ebeaef8e4223"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Power model" sheetId="3" r:id="Ra718c3ec8d094731"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Ra0c72dfe727643a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory" sheetId="2" r:id="Rfb358213ef98485a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Power model" sheetId="3" r:id="Rcd961f9281dd463c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acquisition references" sheetId="4" r:id="Ra97d3b91760b4528"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -118,7 +119,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="48">
+  <x:cellXfs count="53">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -256,6 +257,21 @@
     </x:xf>
     <x:xf numFmtId="202" fontId="1" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="top"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -307,6 +323,22 @@
     <x:tableColumn id="5" name="Working (W)"/>
     <x:tableColumn id="6" name="Heavy (W)"/>
     <x:tableColumn id="7" name="Included equipment and estimate basis"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="RecentAcquisitions" displayName="RecentAcquisitions" ref="A6:G14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A6:G14"/>
+  <x:tableColumns count="7">
+    <x:tableColumn id="1" name="Item ID"/>
+    <x:tableColumn id="2" name="Equipment"/>
+    <x:tableColumn id="3" name="Unit reference (USD)"/>
+    <x:tableColumn id="4" name="Line estimate (USD)"/>
+    <x:tableColumn id="5" name="Power reference"/>
+    <x:tableColumn id="6" name="In current power totals?"/>
+    <x:tableColumn id="7" name="Price and power basis / sources"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -532,7 +564,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="5" t="str">
-        <x:v>Lab inventory, replacement costs and power estimates</x:v>
+        <x:v>Lab inventory, equipment cost and power estimates</x:v>
       </x:c>
       <x:c r="B3" s="5"/>
       <x:c r="C3" s="5"/>
@@ -556,7 +588,7 @@
     </x:row>
     <x:row r="6" ht="38" customHeight="1">
       <x:c r="A6" s="13" t="str">
-        <x:v>Replacement cost estimate</x:v>
+        <x:v>Equipment cost estimate</x:v>
       </x:c>
       <x:c r="B6" s="14" t="str">
         <x:v>USD</x:v>
@@ -568,9 +600,9 @@
       <x:c r="A7" s="3" t="str">
         <x:v>Compute and add-ons</x:v>
       </x:c>
-      <x:c r="B7" s="15" t="str">
+      <x:c r="B7" s="15" t="n">
         <x:f>IF(COUNTIFS('Inventory'!J8:J67,A7,'Inventory'!G8:G67,"Missing input")=0,SUMIFS('Inventory'!G8:G67,'Inventory'!J8:J67,A7),"Missing input")</x:f>
-        <x:v>Missing input</x:v>
+        <x:v>28632</x:v>
       </x:c>
       <x:c r="C7" s="3"/>
       <x:c r="D7" s="3"/>
@@ -579,20 +611,20 @@
       <x:c r="A8" s="3" t="str">
         <x:v>Rack and shared</x:v>
       </x:c>
-      <x:c r="B8" s="15" t="str">
+      <x:c r="B8" s="15" t="n">
         <x:f>IF(COUNTIFS('Inventory'!J8:J67,A8,'Inventory'!G8:G67,"Missing input")=0,SUMIFS('Inventory'!G8:G67,'Inventory'!J8:J67,A8),"Missing input")</x:f>
-        <x:v>Missing input</x:v>
+        <x:v>2613</x:v>
       </x:c>
       <x:c r="C8" s="3"/>
       <x:c r="D8" s="3"/>
     </x:row>
     <x:row r="9" ht="24" customHeight="1">
       <x:c r="A9" s="18" t="str">
-        <x:v>Total replacement estimate</x:v>
-      </x:c>
-      <x:c r="B9" s="19" t="str">
+        <x:v>Total equipment cost estimate</x:v>
+      </x:c>
+      <x:c r="B9" s="19" t="n">
         <x:f>IF(COUNT(B7:B8)=2,SUM(B7:B8),"Missing input")</x:f>
-        <x:v>Missing input</x:v>
+        <x:v>31245</x:v>
       </x:c>
       <x:c r="C9" s="3"/>
       <x:c r="D9" s="3"/>
@@ -603,14 +635,14 @@
       </x:c>
       <x:c r="B10" s="15" t="n">
         <x:f>SUM('Inventory'!G8:G67)</x:f>
-        <x:v>30813</x:v>
+        <x:v>31245</x:v>
       </x:c>
       <x:c r="C10" s="3"/>
       <x:c r="D10" s="3"/>
     </x:row>
     <x:row r="11" ht="24" customHeight="1">
       <x:c r="A11" s="20" t="str">
-        <x:v>Full total needs all prices. Subtotal excludes unpriced equipment; it is not an amount paid.</x:v>
+        <x:v>Dated references and allowances are not the amount paid. Unknown models remain provisional.</x:v>
       </x:c>
       <x:c r="B11" s="3"/>
       <x:c r="C11" s="3"/>
@@ -732,7 +764,7 @@
     </x:row>
     <x:row r="24" ht="24" customHeight="1">
       <x:c r="A24" s="20" t="str">
-        <x:v>Agent Blade watts are projected. Newly acquired equipment is excluded until modeled.</x:v>
+        <x:v>Agent Blade watts are projected. Recent acquisition power is referenced separately.</x:v>
       </x:c>
       <x:c r="B24" s="3"/>
       <x:c r="C24" s="3"/>
@@ -794,7 +826,7 @@
     </x:row>
     <x:row r="32" ht="24" customHeight="1">
       <x:c r="A32" s="20" t="str">
-        <x:v>Reference prices: September 11–12, 2026; reported acquisition costs: September 18.</x:v>
+        <x:v>Original references: September 11–12, 2026; recent acquisition research: September 18.</x:v>
       </x:c>
       <x:c r="B32" s="3"/>
       <x:c r="C32" s="3"/>
@@ -2950,32 +2982,35 @@
       <x:c r="C60" s="38" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D60" s="39"/>
+      <x:c r="D60" s="39" t="n">
+        <x:v>179.99</x:v>
+      </x:c>
       <x:c r="E60" s="39" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F60" s="40" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="G60" s="41" t="str">
+      <x:c r="G60" s="41" t="n">
         <x:f>IF(COUNT(C60:F60)=4,ROUND(C60*(D60+E60),0)+F60,"Missing input")</x:f>
-        <x:v>Missing input</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="H60" s="42" t="str">
         <x:v>none</x:v>
       </x:c>
       <x:c r="I60" s="30" t="str">
-        <x:v>Not modeled: installation and power use unconfirmed</x:v>
+        <x:v>Power reference only; not in configured-lab totals until installed</x:v>
       </x:c>
       <x:c r="J60" s="30" t="str">
         <x:v>Compute and add-ons</x:v>
       </x:c>
       <x:c r="K60" s="3"/>
       <x:c r="L60" s="32" t="str">
-        <x:v>Acquisition reported by Shannon Duncan on September 13, 2026. Installation and availability unconfirmed. No price supplied.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="61" ht="57" customHeight="1">
+        <x:v>Acquired September 13, 2026. Newegg listed a refurbished 8 GB Tesla P4 at $179.99 on September 18. Exact card condition and installation are unconfirmed.
+https://www.newegg.com/p/pl?N=100006519+100&amp;d=nvidia+tesla+p4+8gb</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="91" customHeight="1">
       <x:c r="A61" s="16" t="str">
         <x:v>EQ-54</x:v>
       </x:c>
@@ -3002,17 +3037,19 @@
         <x:v>none</x:v>
       </x:c>
       <x:c r="I61" s="30" t="str">
-        <x:v>Not modeled: replacement of or addition to the existing UPS branch is unconfirmed</x:v>
+        <x:v>UPS overhead reference only; do not add rated output as consumption or double-count the existing UPS</x:v>
       </x:c>
       <x:c r="J61" s="30" t="str">
         <x:v>Rack and shared</x:v>
       </x:c>
       <x:c r="K61" s="3"/>
       <x:c r="L61" s="32" t="str">
-        <x:v>Acquisition and $995 cost reported by Shannon Duncan on September 18, 2026. Its rated output is not a wall-power measurement; installation and overhead are not yet modeled.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="62" ht="57" customHeight="1">
+        <x:v>Shannon reported $995 on September 18, 2026; DigiKey listed the exact model at $995.95. The owner-reported amount is retained as the cost reference. Installation and protected loads are unconfirmed.
+https://www.digikey.com/en/products/detail/cyber-power-systems-usa-inc/PR2200LCDSL/21527902
+https://www.cyberpowersystems.com/product/ups/smart-app-sinewave/pr2200lcdsl/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="77" customHeight="1">
       <x:c r="A62" s="3" t="str">
         <x:v>EQ-55</x:v>
       </x:c>
@@ -3039,14 +3076,15 @@
         <x:v>none</x:v>
       </x:c>
       <x:c r="I62" s="30" t="str">
-        <x:v>Not modeled: bench use and duty cycle unconfirmed</x:v>
+        <x:v>Power reference only; bench duty cycle is not part of current whole-lab scenario</x:v>
       </x:c>
       <x:c r="J62" s="30" t="str">
         <x:v>Compute and add-ons</x:v>
       </x:c>
       <x:c r="K62" s="3"/>
       <x:c r="L62" s="32" t="str">
-        <x:v>Acquisition and $69 cost reported by Shannon Duncan on September 18, 2026. Output rating is not a wall-power measurement.</x:v>
+        <x:v>Shannon reported $69 on September 18, 2026; a current WEP 605D-III listing was $69.98. The owner-reported amount is retained as the cost reference.
+https://www.shopabunda.com/products/wep-605d-iii-dc-variable-power-supply-60-00v-5-000a-high-precision-bench-lab-power-supply-with-alligator-clips-for-anodizing-kit-electroplating-arduino-breadboard</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="57" customHeight="1">
@@ -3059,32 +3097,35 @@
       <x:c r="C63" s="38" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D63" s="39"/>
+      <x:c r="D63" s="39" t="n">
+        <x:v>11.99</x:v>
+      </x:c>
       <x:c r="E63" s="39" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F63" s="40" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="G63" s="41" t="str">
+      <x:c r="G63" s="41" t="n">
         <x:f>IF(COUNT(C63:F63)=4,ROUND(C63*(D63+E63),0)+F63,"Missing input")</x:f>
-        <x:v>Missing input</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="H63" s="42" t="str">
         <x:v>none</x:v>
       </x:c>
       <x:c r="I63" s="30" t="str">
-        <x:v>Not modeled: configuration and active use unconfirmed</x:v>
+        <x:v>Power reference only; configuration and active use unconfirmed</x:v>
       </x:c>
       <x:c r="J63" s="30" t="str">
         <x:v>Compute and add-ons</x:v>
       </x:c>
       <x:c r="K63" s="3"/>
       <x:c r="L63" s="32" t="str">
-        <x:v>Acquisition reported by Shannon Duncan on September 18, 2026. Price, configuration, and active use unconfirmed.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="64" ht="57" customHeight="1">
+        <x:v>Luckfox listed the Mini A base board at $11.99 on September 18, 2026. Flash/header options cost up to $18.99; the acquired variant is not specified.
+https://www.luckfox.com/Luckfox-Pico-Mini-A</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="77" customHeight="1">
       <x:c r="A64" s="3" t="str">
         <x:v>EQ-57</x:v>
       </x:c>
@@ -3094,29 +3135,33 @@
       <x:c r="C64" s="38" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D64" s="39"/>
+      <x:c r="D64" s="39" t="n">
+        <x:v>112.99</x:v>
+      </x:c>
       <x:c r="E64" s="39" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F64" s="40" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="G64" s="41" t="str">
+      <x:c r="G64" s="41" t="n">
         <x:f>IF(COUNT(C64:F64)=4,ROUND(C64*(D64+E64),0)+F64,"Missing input")</x:f>
-        <x:v>Missing input</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="H64" s="42" t="str">
         <x:v>none</x:v>
       </x:c>
       <x:c r="I64" s="30" t="str">
-        <x:v>Not modeled: installation and power use unconfirmed</x:v>
+        <x:v>Provisional Cube-class reference only; variant and installation unconfirmed</x:v>
       </x:c>
       <x:c r="J64" s="30" t="str">
         <x:v>Rack and shared</x:v>
       </x:c>
       <x:c r="K64" s="3"/>
       <x:c r="L64" s="32" t="str">
-        <x:v>Acquisition reported by Shannon Duncan on September 18, 2026. Price and installation unconfirmed.</x:v>
+        <x:v>The exact NanoKVM variant was not specified. A US Cube Full Kit listing was $112.99 on September 18, 2026. This is a provisional comparable reference, not the acquired device's confirmed variant or purchase price; other variants cost less or more.
+https://github.com/sipeed/NanoKVM
+https://www.newegg.com/p/3C6-05G2-02VG1?Item=9SIC5T7KZA4026</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="57" customHeight="1">
@@ -3129,32 +3174,35 @@
       <x:c r="C65" s="38" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D65" s="39"/>
+      <x:c r="D65" s="39" t="n">
+        <x:v>16.99</x:v>
+      </x:c>
       <x:c r="E65" s="39" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F65" s="40" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="G65" s="41" t="str">
+      <x:c r="G65" s="41" t="n">
         <x:f>IF(COUNT(C65:F65)=4,ROUND(C65*(D65+E65),0)+F65,"Missing input")</x:f>
-        <x:v>Missing input</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="H65" s="42" t="str">
         <x:v>none</x:v>
       </x:c>
       <x:c r="I65" s="30" t="str">
-        <x:v>Not modeled: project assignment and active use unconfirmed</x:v>
+        <x:v>Power reference only; camera, host, and deployment configuration unconfirmed</x:v>
       </x:c>
       <x:c r="J65" s="30" t="str">
         <x:v>Compute and add-ons</x:v>
       </x:c>
       <x:c r="K65" s="3"/>
       <x:c r="L65" s="32" t="str">
-        <x:v>Acquisition reported by Shannon Duncan on September 18, 2026. Price and project assignment unconfirmed.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="66" ht="57" customHeight="1">
+        <x:v>Seeed Studio listed the bare Grove Vision AI Module V2 at $16.99 on September 18, 2026. A camera or host board is not included in this line.
+https://www.seeedstudio.com/Grove-Vision-AI-Module-V2-p-5851.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="63" customHeight="1">
       <x:c r="A66" s="3" t="str">
         <x:v>EQ-59</x:v>
       </x:c>
@@ -3164,32 +3212,35 @@
       <x:c r="C66" s="38" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D66" s="39"/>
+      <x:c r="D66" s="39" t="n">
+        <x:v>49.99</x:v>
+      </x:c>
       <x:c r="E66" s="39" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F66" s="40" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="G66" s="41" t="str">
+      <x:c r="G66" s="41" t="n">
         <x:f>IF(COUNT(C66:F66)=4,ROUND(C66*(D66+E66),0)+F66,"Missing input")</x:f>
-        <x:v>Missing input</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="H66" s="42" t="str">
         <x:v>none</x:v>
       </x:c>
       <x:c r="I66" s="30" t="str">
-        <x:v>Not modeled: model and duty cycle unconfirmed</x:v>
+        <x:v>Power reference only; model and bench duty cycle unconfirmed</x:v>
       </x:c>
       <x:c r="J66" s="30" t="str">
         <x:v>Compute and add-ons</x:v>
       </x:c>
       <x:c r="K66" s="3"/>
       <x:c r="L66" s="32" t="str">
-        <x:v>Acquisition reported by Shannon Duncan on September 18, 2026. Model, price, and active power use unconfirmed.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="67" ht="57" customHeight="1">
+        <x:v>The acquired setup's make and contents were not specified. iFixit's entry-level soldering workstation was $49.99 on September 18, 2026; this is a comparable allowance, not the actual paid price or an exact replacement match.
+https://www.ifixit.com/products/soldering-workstation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="63" customHeight="1">
       <x:c r="A67" s="16" t="str">
         <x:v>EQ-60</x:v>
       </x:c>
@@ -3199,29 +3250,32 @@
       <x:c r="C67" s="38" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D67" s="39"/>
+      <x:c r="D67" s="39" t="n">
+        <x:v>59.9</x:v>
+      </x:c>
       <x:c r="E67" s="39" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F67" s="40" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="G67" s="41" t="str">
+      <x:c r="G67" s="41" t="n">
         <x:f>IF(COUNT(C67:F67)=4,ROUND(C67*(D67+E67),0)+F67,"Missing input")</x:f>
-        <x:v>Missing input</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="H67" s="42" t="str">
         <x:v>none</x:v>
       </x:c>
       <x:c r="I67" s="30" t="str">
-        <x:v>Not modeled: project assignment and active use unconfirmed</x:v>
+        <x:v>Power reference only; do not double-count the existing M5Stack power group until quantity is confirmed</x:v>
       </x:c>
       <x:c r="J67" s="30" t="str">
         <x:v>Compute and add-ons</x:v>
       </x:c>
       <x:c r="K67" s="3"/>
       <x:c r="L67" s="32" t="str">
-        <x:v>Acquisition reported by Shannon Duncan on September 18, 2026. Price and project assignment unconfirmed.</x:v>
+        <x:v>M5Stack listed the CoreS3 IoT development kit at $59.90 on September 18, 2026. The older registry also has one M5Stack ESP32-S3 device (EQ-29); this line assumes the newly reported CoreS3 is additional until the owner confirms whether it is the same unit.
+https://shop.m5stack.com/products/m5stack-cores3-esp32s3-iotdevelopment-kit</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="24" customHeight="1">
@@ -3240,16 +3294,16 @@
     </x:row>
     <x:row r="69" ht="30" customHeight="1">
       <x:c r="A69" s="18" t="str">
-        <x:v>Total replacement estimate</x:v>
+        <x:v>Total equipment cost estimate</x:v>
       </x:c>
       <x:c r="B69" s="18"/>
       <x:c r="C69" s="18"/>
       <x:c r="D69" s="18"/>
       <x:c r="E69" s="18"/>
       <x:c r="F69" s="18"/>
-      <x:c r="G69" s="19" t="str">
+      <x:c r="G69" s="19" t="n">
         <x:f>IF(COUNT(G8:G67)=ROWS(G8:G67),SUM(G8:G67),"Missing input")</x:f>
-        <x:v>Missing input</x:v>
+        <x:v>31245</x:v>
       </x:c>
       <x:c r="H69" s="18"/>
       <x:c r="I69" s="18"/>
@@ -3313,7 +3367,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R650c21c70b554253"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R78956d59cc9043be"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4157,7 +4211,365 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbf31bd9d29d5407b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re0e46ee680c049a6"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FFFF553D"/>
+  </x:sheetPr>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="13" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="50" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="17" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="58" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="27" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="95" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="24" customHeight="1">
+      <x:c r="A1" s="3"/>
+      <x:c r="B1" s="3"/>
+      <x:c r="C1" s="3"/>
+      <x:c r="D1" s="3"/>
+      <x:c r="E1" s="3"/>
+      <x:c r="F1" s="3"/>
+      <x:c r="G1" s="3"/>
+    </x:row>
+    <x:row r="2" ht="24" customHeight="1">
+      <x:c r="A2" s="4" t="str">
+        <x:v>Recent acquisition references</x:v>
+      </x:c>
+      <x:c r="B2" s="3"/>
+      <x:c r="C2" s="3"/>
+      <x:c r="D2" s="3"/>
+      <x:c r="E2" s="3"/>
+      <x:c r="F2" s="3"/>
+      <x:c r="G2" s="3"/>
+    </x:row>
+    <x:row r="3" ht="24" customHeight="1">
+      <x:c r="A3" s="20" t="str">
+        <x:v>Prices are dated replacement references or explicit allowances, not necessarily purchase costs.</x:v>
+      </x:c>
+      <x:c r="B3" s="3"/>
+      <x:c r="C3" s="3"/>
+      <x:c r="D3" s="3"/>
+      <x:c r="E3" s="3"/>
+      <x:c r="F3" s="3"/>
+      <x:c r="G3" s="3"/>
+    </x:row>
+    <x:row r="4" ht="24" customHeight="1">
+      <x:c r="A4" s="20" t="str">
+        <x:v>Power figures describe the device or output, as noted. None is added to the current configured-lab totals.</x:v>
+      </x:c>
+      <x:c r="B4" s="3"/>
+      <x:c r="C4" s="3"/>
+      <x:c r="D4" s="3"/>
+      <x:c r="E4" s="3"/>
+      <x:c r="F4" s="3"/>
+      <x:c r="G4" s="3"/>
+    </x:row>
+    <x:row r="5" ht="24" customHeight="1">
+      <x:c r="A5" s="3"/>
+      <x:c r="B5" s="3"/>
+      <x:c r="C5" s="3"/>
+      <x:c r="D5" s="3"/>
+      <x:c r="E5" s="3"/>
+      <x:c r="F5" s="3"/>
+      <x:c r="G5" s="3"/>
+    </x:row>
+    <x:row r="6" ht="38" customHeight="1">
+      <x:c r="A6" s="13" t="str">
+        <x:v>Item ID</x:v>
+      </x:c>
+      <x:c r="B6" s="23" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="C6" s="23" t="str">
+        <x:v>Unit reference (USD)</x:v>
+      </x:c>
+      <x:c r="D6" s="23" t="str">
+        <x:v>Line estimate (USD)</x:v>
+      </x:c>
+      <x:c r="E6" s="23" t="str">
+        <x:v>Power reference</x:v>
+      </x:c>
+      <x:c r="F6" s="23" t="str">
+        <x:v>In current power totals?</x:v>
+      </x:c>
+      <x:c r="G6" s="14" t="str">
+        <x:v>Price and power basis / sources</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="135" customHeight="1">
+      <x:c r="A7" s="49" t="str">
+        <x:v>EQ-53</x:v>
+      </x:c>
+      <x:c r="B7" s="51" t="str">
+        <x:v>NVIDIA P4 GPU, 8 GB memory</x:v>
+      </x:c>
+      <x:c r="C7" s="52" t="n">
+        <x:f>Inventory!D60</x:f>
+        <x:v>179.99</x:v>
+      </x:c>
+      <x:c r="D7" s="52" t="n">
+        <x:f>Inventory!G60</x:f>
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="E7" s="51" t="str">
+        <x:v>50 or 75 W board-power design; idle draw and host overhead unknown</x:v>
+      </x:c>
+      <x:c r="F7" s="51" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="G7" s="51" t="str">
+        <x:v>Dated refurbished replacement reference. Acquired September 13, 2026. Newegg listed a refurbished 8 GB Tesla P4 at $179.99 on September 18. Exact card condition and installation are unconfirmed.
+Price: https://www.newegg.com/p/pl?N=100006519+100&amp;d=nvidia+tesla+p4+8gb
+Power: NVIDIA Tesla P4 datasheet. These are design power options, not measured draw for this card.
+https://www.nvidia.com/content/dam/en-zz/Solutions/Data-Center/tesla-product-literature/184457-Tesla-P4-Datasheet-NV-Final-Letter-Web.pdf</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="135" customHeight="1">
+      <x:c r="A8" s="49" t="str">
+        <x:v>EQ-54</x:v>
+      </x:c>
+      <x:c r="B8" s="51" t="str">
+        <x:v>CyberPower PR2200LCDSL Smart App Sinewave UPS, 2070 VA / 1980 W, 7 outlets, AVR, mini-tower</x:v>
+      </x:c>
+      <x:c r="C8" s="52" t="n">
+        <x:f>Inventory!D61</x:f>
+        <x:v>995</x:v>
+      </x:c>
+      <x:c r="D8" s="52" t="n">
+        <x:f>Inventory!G61</x:f>
+        <x:v>995</x:v>
+      </x:c>
+      <x:c r="E8" s="51" t="str">
+        <x:v>6 W at no load; about 98% efficient at 25% output load and 99% at 50%</x:v>
+      </x:c>
+      <x:c r="F8" s="51" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="G8" s="51" t="str">
+        <x:v>Owner-reported price, checked against current listing. Shannon reported $995 on September 18, 2026; DigiKey listed the exact model at $995.95. The owner-reported amount is retained as the cost reference. Installation and protected loads are unconfirmed.
+Price: https://www.digikey.com/en/products/detail/cyber-power-systems-usa-inc/PR2200LCDSL/21527902 | https://www.cyberpowersystems.com/product/ups/smart-app-sinewave/pr2200lcdsl/
+Power: ENERGY STAR test for PR2200LCDSL. Output capacity is 1,980 W, not wall draw. Overhead depends on attached load and whether this UPS replaces or supplements the 750 VA unit; battery recharge is excluded.
+https://downloads.energystar.gov/bi/qplist/Uninterruptible_Power_Supplies_Product_List.pdf</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="135" customHeight="1">
+      <x:c r="A9" s="49" t="str">
+        <x:v>EQ-55</x:v>
+      </x:c>
+      <x:c r="B9" s="51" t="str">
+        <x:v>WEP 605D-III DC variable bench power supply, 60 V / 5 A</x:v>
+      </x:c>
+      <x:c r="C9" s="52" t="n">
+        <x:f>Inventory!D62</x:f>
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="D9" s="52" t="n">
+        <x:f>Inventory!G62</x:f>
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="E9" s="51" t="str">
+        <x:v>Up to 300 W DC output; roughly 375 W AC input at full output if efficiency is 80%</x:v>
+      </x:c>
+      <x:c r="F9" s="51" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="G9" s="51" t="str">
+        <x:v>Owner-reported price, checked against current listing. Shannon reported $69 on September 18, 2026; a current WEP 605D-III listing was $69.98. The owner-reported amount is retained as the cost reference.
+Price: https://www.shopabunda.com/products/wep-605d-iii-dc-variable-power-supply-60-00v-5-000a-high-precision-bench-lab-power-supply-with-alligator-clips-for-anodizing-kit-electroplating-arduino-breadboard
+Power: 60 V × 5 A gives 300 W maximum output. The 80% conversion-efficiency assumption comes from a comparable 60 V / 5 A bench supply, not a published WEP measurement. Actual wall draw follows the connected load.
+https://www.farnell.com/datasheets/4459704.pdf</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="135" customHeight="1">
+      <x:c r="A10" s="49" t="str">
+        <x:v>EQ-56</x:v>
+      </x:c>
+      <x:c r="B10" s="51" t="str">
+        <x:v>Luckfox Pico Mini A</x:v>
+      </x:c>
+      <x:c r="C10" s="52" t="n">
+        <x:f>Inventory!D63</x:f>
+        <x:v>11.99</x:v>
+      </x:c>
+      <x:c r="D10" s="52" t="n">
+        <x:f>Inventory!G63</x:f>
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E10" s="51" t="str">
+        <x:v>About 1-2 W planning allowance when powered by USB-C; no model-specific draw published</x:v>
+      </x:c>
+      <x:c r="F10" s="51" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="G10" s="51" t="str">
+        <x:v>Dated base-variant price reference. Luckfox listed the Mini A base board at $11.99 on September 18, 2026. Flash/header options cost up to $18.99; the acquired variant is not specified.
+Price: https://www.luckfox.com/Luckfox-Pico-Mini-A
+Power: Luckfox documents USB-C power but does not publish a board-level watt figure. This is an explicit low-power board allowance, not a measured specification; connected USB peripherals and cameras add load.
+https://www.luckfox.com/Luckfox-Pico-Mini-A</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="135" customHeight="1">
+      <x:c r="A11" s="49" t="str">
+        <x:v>EQ-57</x:v>
+      </x:c>
+      <x:c r="B11" s="51" t="str">
+        <x:v>Sipeed NanoKVM</x:v>
+      </x:c>
+      <x:c r="C11" s="52" t="n">
+        <x:f>Inventory!D64</x:f>
+        <x:v>112.99</x:v>
+      </x:c>
+      <x:c r="D11" s="52" t="n">
+        <x:f>Inventory!G64</x:f>
+        <x:v>113</x:v>
+      </x:c>
+      <x:c r="E11" s="51" t="str">
+        <x:v>About 1 W for NanoKVM Cube; other NanoKVM variants can differ</x:v>
+      </x:c>
+      <x:c r="F11" s="51" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="G11" s="51" t="str">
+        <x:v>Provisional Cube Full-class US replacement reference. The exact NanoKVM variant was not specified. A US Cube Full Kit listing was $112.99 on September 18, 2026. This is a provisional comparable reference, not the acquired device's confirmed variant or purchase price; other variants cost less or more.
+Price: https://github.com/sipeed/NanoKVM | https://www.newegg.com/p/3C6-05G2-02VG1?Item=9SIC5T7KZA4026
+Power: Sipeed's NanoKVM Cube quick-start states about 1 W at 5 V. This cannot be treated as the acquired device's draw until the variant is identified.
+https://wiki.sipeed.com/hardware/en/kvm/NanoKVM/quick_start.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="135" customHeight="1">
+      <x:c r="A12" s="49" t="str">
+        <x:v>EQ-58</x:v>
+      </x:c>
+      <x:c r="B12" s="51" t="str">
+        <x:v>Grove Vision AI Module V2</x:v>
+      </x:c>
+      <x:c r="C12" s="52" t="n">
+        <x:f>Inventory!D65</x:f>
+        <x:v>16.99</x:v>
+      </x:c>
+      <x:c r="D12" s="52" t="n">
+        <x:f>Inventory!G65</x:f>
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="E12" s="51" t="str">
+        <x:v>About 0.35-0.42 W during published inference examples; host and camera separate</x:v>
+      </x:c>
+      <x:c r="F12" s="51" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="G12" s="51" t="str">
+        <x:v>Dated manufacturer price reference. Seeed Studio listed the bare Grove Vision AI Module V2 at $16.99 on September 18, 2026. A camera or host board is not included in this line.
+Price: https://www.seeedstudio.com/Grove-Vision-AI-Module-V2-p-5851.html
+Power: Published tests report about 0.35 W average and 0.42 W peak for specific vision workloads. This is not a site measurement and is not a universal maximum.
+https://www.hackster.io/limengdu0117/2024-mcu-ai-vision-boards-performance-comparison-998505 | https://mlsysbook.ai/kits/contents/seeed/grove_vision_ai_v2/setup_and_no_code_apps/setup_and_no_code_apps.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="135" customHeight="1">
+      <x:c r="A13" s="49" t="str">
+        <x:v>EQ-59</x:v>
+      </x:c>
+      <x:c r="B13" s="51" t="str">
+        <x:v>Soldering iron setup</x:v>
+      </x:c>
+      <x:c r="C13" s="52" t="n">
+        <x:f>Inventory!D66</x:f>
+        <x:v>49.99</x:v>
+      </x:c>
+      <x:c r="D13" s="52" t="n">
+        <x:f>Inventory!G66</x:f>
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="E13" s="51" t="str">
+        <x:v>About 30-60 W while heating for a 60 W-class iron; near zero unplugged</x:v>
+      </x:c>
+      <x:c r="F13" s="51" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="G13" s="51" t="str">
+        <x:v>Provisional comparable-kit allowance. The acquired setup's make and contents were not specified. iFixit's entry-level soldering workstation was $49.99 on September 18, 2026; this is a comparable allowance, not the actual paid price or an exact replacement match.
+Price: https://www.ifixit.com/products/soldering-workstation
+Power: Comparable 60 W soldering irons are load- and thermostat-dependent. This is a planning range, not a specification for the acquired setup; hot-air stations may draw much more.
+https://www.adafruit.com/explore/tools</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="135" customHeight="1">
+      <x:c r="A14" s="49" t="str">
+        <x:v>EQ-60</x:v>
+      </x:c>
+      <x:c r="B14" s="51" t="str">
+        <x:v>M5Stack CoreS3 ESP32-S3 development kit</x:v>
+      </x:c>
+      <x:c r="C14" s="52" t="n">
+        <x:f>Inventory!D67</x:f>
+        <x:v>59.9</x:v>
+      </x:c>
+      <x:c r="D14" s="52" t="n">
+        <x:f>Inventory!G67</x:f>
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="E14" s="51" t="str">
+        <x:v>About 1.5-3 W planning range when active; peripherals and charging vary</x:v>
+      </x:c>
+      <x:c r="F14" s="51" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="G14" s="51" t="str">
+        <x:v>Dated manufacturer price reference. M5Stack listed the CoreS3 IoT development kit at $59.90 on September 18, 2026. The older registry also has one M5Stack ESP32-S3 device (EQ-29); this line assumes the newly reported CoreS3 is additional until the owner confirms whether it is the same unit.
+Price: https://shop.m5stack.com/products/m5stack-cores3-esp32s3-iotdevelopment-kit
+Power: Uses the existing M5Stack ESP32-S3 bench allowance as a comparable reference. The CoreS3 has a battery and 1 W speaker; manufacturer does not publish a whole-kit wall-power measurement. Additional-unit status is unconfirmed.
+https://shop.m5stack.com/products/m5stack-cores3-esp32s3-iotdevelopment-kit</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="24" customHeight="1">
+      <x:c r="A15" s="3"/>
+      <x:c r="B15" s="3"/>
+      <x:c r="C15" s="3"/>
+      <x:c r="D15" s="3"/>
+      <x:c r="E15" s="3"/>
+      <x:c r="F15" s="3"/>
+      <x:c r="G15" s="3"/>
+    </x:row>
+    <x:row r="16" ht="24" customHeight="1">
+      <x:c r="A16" s="3"/>
+      <x:c r="B16" s="3"/>
+      <x:c r="C16" s="3"/>
+      <x:c r="D16" s="3"/>
+      <x:c r="E16" s="3"/>
+      <x:c r="F16" s="3"/>
+      <x:c r="G16" s="3"/>
+    </x:row>
+    <x:row r="17" ht="24" customHeight="1">
+      <x:c r="A17" s="3"/>
+      <x:c r="B17" s="3"/>
+      <x:c r="C17" s="3"/>
+      <x:c r="D17" s="3"/>
+      <x:c r="E17" s="3"/>
+      <x:c r="F17" s="3"/>
+      <x:c r="G17" s="3"/>
+    </x:row>
+    <x:row r="18" ht="24" customHeight="1">
+      <x:c r="A18" s="3"/>
+      <x:c r="B18" s="3"/>
+      <x:c r="C18" s="3"/>
+      <x:c r="D18" s="3"/>
+      <x:c r="E18" s="3"/>
+      <x:c r="F18" s="3"/>
+      <x:c r="G18" s="3"/>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf832c33745a94a08"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Make free Lab compute clear and record new GPU acquisitions
</commit_message>
<xml_diff>
--- a/public/lab/hack-lab-inventory.xlsx
+++ b/public/lab/hack-lab-inventory.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Ra0c72dfe727643a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory" sheetId="2" r:id="Rfb358213ef98485a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Power model" sheetId="3" r:id="Rcd961f9281dd463c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acquisition references" sheetId="4" r:id="Ra97d3b91760b4528"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R7f7b50554c954ee0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory" sheetId="2" r:id="Ra10e0dd746a14ef2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Power model" sheetId="3" r:id="R7b2434715ba344c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device references" sheetId="4" r:id="Rad036bf103cb4bdb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -294,8 +294,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="LabInventory" displayName="LabInventory" ref="A7:J67" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A7:J67"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="LabInventory" displayName="LabInventory" ref="A7:J70" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A7:J70"/>
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="Item ID"/>
     <x:tableColumn id="2" name="Equipment and specifications"/>
@@ -329,8 +329,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="RecentAcquisitions" displayName="RecentAcquisitions" ref="A6:G14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A6:G14"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DeviceReferences" displayName="DeviceReferences" ref="A6:G17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A6:G17"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="Item ID"/>
     <x:tableColumn id="2" name="Equipment"/>
@@ -575,7 +575,7 @@
         <x:v>Snapshot</x:v>
       </x:c>
       <x:c r="B4" s="6" t="n">
-        <x:v>46283.5</x:v>
+        <x:v>46288.5</x:v>
       </x:c>
       <x:c r="C4" s="3"/>
       <x:c r="D4" s="3"/>
@@ -601,8 +601,8 @@
         <x:v>Compute and add-ons</x:v>
       </x:c>
       <x:c r="B7" s="15" t="n">
-        <x:f>IF(COUNTIFS('Inventory'!J8:J67,A7,'Inventory'!G8:G67,"Missing input")=0,SUMIFS('Inventory'!G8:G67,'Inventory'!J8:J67,A7),"Missing input")</x:f>
-        <x:v>28632</x:v>
+        <x:f>IF(COUNTIFS('Inventory'!J8:J70,A7,'Inventory'!G8:G70,"Missing input")=0,SUMIFS('Inventory'!G8:G70,'Inventory'!J8:J70,A7),"Missing input")</x:f>
+        <x:v>32331</x:v>
       </x:c>
       <x:c r="C7" s="3"/>
       <x:c r="D7" s="3"/>
@@ -612,7 +612,7 @@
         <x:v>Rack and shared</x:v>
       </x:c>
       <x:c r="B8" s="15" t="n">
-        <x:f>IF(COUNTIFS('Inventory'!J8:J67,A8,'Inventory'!G8:G67,"Missing input")=0,SUMIFS('Inventory'!G8:G67,'Inventory'!J8:J67,A8),"Missing input")</x:f>
+        <x:f>IF(COUNTIFS('Inventory'!J8:J70,A8,'Inventory'!G8:G70,"Missing input")=0,SUMIFS('Inventory'!G8:G70,'Inventory'!J8:J70,A8),"Missing input")</x:f>
         <x:v>2613</x:v>
       </x:c>
       <x:c r="C8" s="3"/>
@@ -624,7 +624,7 @@
       </x:c>
       <x:c r="B9" s="19" t="n">
         <x:f>IF(COUNT(B7:B8)=2,SUM(B7:B8),"Missing input")</x:f>
-        <x:v>31245</x:v>
+        <x:v>34944</x:v>
       </x:c>
       <x:c r="C9" s="3"/>
       <x:c r="D9" s="3"/>
@@ -634,8 +634,8 @@
         <x:v>Priced equipment subtotal</x:v>
       </x:c>
       <x:c r="B10" s="15" t="n">
-        <x:f>SUM('Inventory'!G8:G67)</x:f>
-        <x:v>31245</x:v>
+        <x:f>SUM('Inventory'!G8:G70)</x:f>
+        <x:v>34944</x:v>
       </x:c>
       <x:c r="C10" s="3"/>
       <x:c r="D10" s="3"/>
@@ -764,7 +764,7 @@
     </x:row>
     <x:row r="24" ht="24" customHeight="1">
       <x:c r="A24" s="20" t="str">
-        <x:v>Agent Blade watts are projected. Recent acquisition power is referenced separately.</x:v>
+        <x:v>Agent Blade watts are projected. Unmodeled devices have separate power references.</x:v>
       </x:c>
       <x:c r="B24" s="3"/>
       <x:c r="C24" s="3"/>
@@ -826,7 +826,7 @@
     </x:row>
     <x:row r="32" ht="24" customHeight="1">
       <x:c r="A32" s="20" t="str">
-        <x:v>Original references: September 11–12, 2026; recent acquisition research: September 18.</x:v>
+        <x:v>Original references: September 11–12, 2026; added devices researched through September 23.</x:v>
       </x:c>
       <x:c r="B32" s="3"/>
       <x:c r="C32" s="3"/>
@@ -935,7 +935,7 @@
     </x:row>
     <x:row r="5" ht="24" customHeight="1">
       <x:c r="A5" s="20" t="str">
-        <x:v>Blank costs are unknown, not zero. Newly acquired equipment has its status in the source note.</x:v>
+        <x:v>Blank costs are unknown, not zero. Source notes distinguish dated prices and provisional allowances.</x:v>
       </x:c>
       <x:c r="B5" s="3"/>
       <x:c r="C5" s="3"/>
@@ -3278,52 +3278,119 @@
 https://shop.m5stack.com/products/m5stack-cores3-esp32s3-iotdevelopment-kit</x:v>
       </x:c>
     </x:row>
-    <x:row r="68" ht="24" customHeight="1">
-      <x:c r="A68" s="3"/>
-      <x:c r="B68" s="3"/>
-      <x:c r="C68" s="3"/>
-      <x:c r="D68" s="3"/>
-      <x:c r="E68" s="3"/>
-      <x:c r="F68" s="3"/>
-      <x:c r="G68" s="3"/>
-      <x:c r="H68" s="3"/>
-      <x:c r="I68" s="3"/>
-      <x:c r="J68" s="3"/>
+    <x:row r="68" ht="91" customHeight="1">
+      <x:c r="A68" s="3" t="str">
+        <x:v>EQ-61</x:v>
+      </x:c>
+      <x:c r="B68" s="30" t="str">
+        <x:v>NVIDIA GeForce RTX 5070, 12 GB GDDR7</x:v>
+      </x:c>
+      <x:c r="C68" s="38" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D68" s="39" t="n">
+        <x:v>799.99</x:v>
+      </x:c>
+      <x:c r="E68" s="39" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F68" s="40" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G68" s="41" t="n">
+        <x:f>IF(COUNT(C68:F68)=4,ROUND(C68*(D68+E68),0)+F68,"Missing input")</x:f>
+        <x:v>1600</x:v>
+      </x:c>
+      <x:c r="H68" s="42" t="str">
+        <x:v>none</x:v>
+      </x:c>
+      <x:c r="I68" s="30" t="str">
+        <x:v>Two acquired cards; installation and simultaneous use unconfirmed. Excluded from current V100 dock scenario</x:v>
+      </x:c>
+      <x:c r="J68" s="30" t="str">
+        <x:v>Compute and add-ons</x:v>
+      </x:c>
       <x:c r="K68" s="3"/>
-      <x:c r="L68" s="3"/>
-    </x:row>
-    <x:row r="69" ht="30" customHeight="1">
-      <x:c r="A69" s="18" t="str">
-        <x:v>Total equipment cost estimate</x:v>
-      </x:c>
-      <x:c r="B69" s="18"/>
-      <x:c r="C69" s="18"/>
-      <x:c r="D69" s="18"/>
-      <x:c r="E69" s="18"/>
-      <x:c r="F69" s="18"/>
-      <x:c r="G69" s="19" t="n">
-        <x:f>IF(COUNT(G8:G67)=ROWS(G8:G67),SUM(G8:G67),"Missing input")</x:f>
-        <x:v>31245</x:v>
-      </x:c>
-      <x:c r="H69" s="18"/>
-      <x:c r="I69" s="18"/>
-      <x:c r="J69" s="18"/>
+      <x:c r="L68" s="32" t="str">
+        <x:v>Acquired and reported September 23, 2026. Exact board makers and purchase prices were not supplied. Best Buy listed a PNY RTX 5070 12 GB card for $799.99 each; two comparable cards are used for this planning estimate. Actual card specifications and availability may differ.
+https://www.bestbuy.com/product/pny-geforce-rtx-5070-12gb-oc-gddr7-pci-express-5-0-graphics-card-with-triple-fan-black/6620352</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69" ht="63" customHeight="1">
+      <x:c r="A69" s="16" t="str">
+        <x:v>EQ-62</x:v>
+      </x:c>
+      <x:c r="B69" s="43" t="str">
+        <x:v>NVIDIA GeForce RTX 4070 SUPER, 12 GB GDDR6X</x:v>
+      </x:c>
+      <x:c r="C69" s="38" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D69" s="39" t="n">
+        <x:v>799</x:v>
+      </x:c>
+      <x:c r="E69" s="39" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F69" s="40" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G69" s="41" t="n">
+        <x:f>IF(COUNT(C69:F69)=4,ROUND(C69*(D69+E69),0)+F69,"Missing input")</x:f>
+        <x:v>799</x:v>
+      </x:c>
+      <x:c r="H69" s="42" t="str">
+        <x:v>none</x:v>
+      </x:c>
+      <x:c r="I69" s="30" t="str">
+        <x:v>Acquired swap card; installation unconfirmed. Excluded from current V100 dock scenario</x:v>
+      </x:c>
+      <x:c r="J69" s="30" t="str">
+        <x:v>Compute and add-ons</x:v>
+      </x:c>
       <x:c r="K69" s="3"/>
-      <x:c r="L69" s="3"/>
-    </x:row>
-    <x:row r="70" ht="24" customHeight="1">
-      <x:c r="A70" s="3"/>
-      <x:c r="B70" s="3"/>
-      <x:c r="C70" s="3"/>
-      <x:c r="D70" s="3"/>
-      <x:c r="E70" s="3"/>
-      <x:c r="F70" s="3"/>
-      <x:c r="G70" s="3"/>
-      <x:c r="H70" s="3"/>
-      <x:c r="I70" s="3"/>
-      <x:c r="J70" s="3"/>
+      <x:c r="L69" s="32" t="str">
+        <x:v>Acquired and reported September 23, 2026. Exact board maker and purchase price were not supplied. Walmart listed a PNY RTX 4070 SUPER 12 GB for $799.00; this is a comparable planning reference.
+https://www.walmart.com/ip/5265483626</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70" ht="91" customHeight="1">
+      <x:c r="A70" s="3" t="str">
+        <x:v>EQ-63</x:v>
+      </x:c>
+      <x:c r="B70" s="30" t="str">
+        <x:v>Intel Arc Pro B70, 32 GB GDDR6</x:v>
+      </x:c>
+      <x:c r="C70" s="38" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D70" s="39" t="n">
+        <x:v>1299.99</x:v>
+      </x:c>
+      <x:c r="E70" s="39" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F70" s="40" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G70" s="41" t="n">
+        <x:f>IF(COUNT(C70:F70)=4,ROUND(C70*(D70+E70),0)+F70,"Missing input")</x:f>
+        <x:v>1300</x:v>
+      </x:c>
+      <x:c r="H70" s="42" t="str">
+        <x:v>none</x:v>
+      </x:c>
+      <x:c r="I70" s="30" t="str">
+        <x:v>Acquired card; exact board and installation unconfirmed. Excluded from current V100 dock scenario</x:v>
+      </x:c>
+      <x:c r="J70" s="30" t="str">
+        <x:v>Compute and add-ons</x:v>
+      </x:c>
       <x:c r="K70" s="3"/>
-      <x:c r="L70" s="3"/>
+      <x:c r="L70" s="32" t="str">
+        <x:v>Acquired and reported September 23, 2026 as a B70. This registry assumes Intel Arc Pro B70; the exact board maker and paid price were not supplied. Newegg listed an ASRock Arc Pro B70 CT 32 GB for $1,299.99. The listing is a comparable replacement reference, not an identification of the acquired card.
+https://www.newegg.com/asrock-b70-ct-intel-arc-pro-b70-32gb-graphics-card/p/N82E16814930149</x:v>
+      </x:c>
     </x:row>
     <x:row r="71" ht="24" customHeight="1">
       <x:c r="A71" s="3"/>
@@ -3339,35 +3406,82 @@
       <x:c r="K71" s="3"/>
       <x:c r="L71" s="3"/>
     </x:row>
-    <x:row r="72" ht="24" customHeight="1">
-      <x:c r="A72" s="3"/>
-      <x:c r="B72" s="3"/>
-      <x:c r="C72" s="3"/>
-      <x:c r="D72" s="3"/>
-      <x:c r="E72" s="3"/>
-      <x:c r="F72" s="3"/>
-      <x:c r="G72" s="3"/>
-      <x:c r="H72" s="3"/>
-      <x:c r="I72" s="3"/>
-      <x:c r="J72" s="3"/>
+    <x:row r="72" ht="30" customHeight="1">
+      <x:c r="A72" s="18" t="str">
+        <x:v>Total equipment cost estimate</x:v>
+      </x:c>
+      <x:c r="B72" s="18"/>
+      <x:c r="C72" s="18"/>
+      <x:c r="D72" s="18"/>
+      <x:c r="E72" s="18"/>
+      <x:c r="F72" s="18"/>
+      <x:c r="G72" s="19" t="n">
+        <x:f>IF(COUNT(G8:G70)=ROWS(G8:G70),SUM(G8:G70),"Missing input")</x:f>
+        <x:v>34944</x:v>
+      </x:c>
+      <x:c r="H72" s="18"/>
+      <x:c r="I72" s="18"/>
+      <x:c r="J72" s="18"/>
       <x:c r="K72" s="3"/>
       <x:c r="L72" s="3"/>
     </x:row>
+    <x:row r="73" ht="24" customHeight="1">
+      <x:c r="A73" s="3"/>
+      <x:c r="B73" s="3"/>
+      <x:c r="C73" s="3"/>
+      <x:c r="D73" s="3"/>
+      <x:c r="E73" s="3"/>
+      <x:c r="F73" s="3"/>
+      <x:c r="G73" s="3"/>
+      <x:c r="H73" s="3"/>
+      <x:c r="I73" s="3"/>
+      <x:c r="J73" s="3"/>
+      <x:c r="K73" s="3"/>
+      <x:c r="L73" s="3"/>
+    </x:row>
+    <x:row r="74" ht="24" customHeight="1">
+      <x:c r="A74" s="3"/>
+      <x:c r="B74" s="3"/>
+      <x:c r="C74" s="3"/>
+      <x:c r="D74" s="3"/>
+      <x:c r="E74" s="3"/>
+      <x:c r="F74" s="3"/>
+      <x:c r="G74" s="3"/>
+      <x:c r="H74" s="3"/>
+      <x:c r="I74" s="3"/>
+      <x:c r="J74" s="3"/>
+      <x:c r="K74" s="3"/>
+      <x:c r="L74" s="3"/>
+    </x:row>
+    <x:row r="75" ht="24" customHeight="1">
+      <x:c r="A75" s="3"/>
+      <x:c r="B75" s="3"/>
+      <x:c r="C75" s="3"/>
+      <x:c r="D75" s="3"/>
+      <x:c r="E75" s="3"/>
+      <x:c r="F75" s="3"/>
+      <x:c r="G75" s="3"/>
+      <x:c r="H75" s="3"/>
+      <x:c r="I75" s="3"/>
+      <x:c r="J75" s="3"/>
+      <x:c r="K75" s="3"/>
+      <x:c r="L75" s="3"/>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="G8:G67">
+  <x:conditionalFormatting sqref="G8:G70">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Missing input"/>
   </x:conditionalFormatting>
   <x:dataValidations count="2">
-    <x:dataValidation type="whole" operator="greaterThanOrEqual" sqref="C8:C67">
+    <x:dataValidation type="whole" operator="greaterThanOrEqual" sqref="C8:C70">
       <x:formula1>0</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="decimal" operator="greaterThanOrEqual" sqref="D8:E67">
+    <x:dataValidation type="decimal" operator="greaterThanOrEqual" sqref="D8:E70">
       <x:formula1>0</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R78956d59cc9043be"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26e774bc00c84f92"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4211,7 +4325,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re0e46ee680c049a6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R60913cfa222a4280"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4243,7 +4357,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="4" t="str">
-        <x:v>Recent acquisition references</x:v>
+        <x:v>Device cost and power references</x:v>
       </x:c>
       <x:c r="B2" s="3"/>
       <x:c r="C2" s="3"/>
@@ -4530,32 +4644,89 @@
 https://shop.m5stack.com/products/m5stack-cores3-esp32s3-iotdevelopment-kit</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="24" customHeight="1">
-      <x:c r="A15" s="3"/>
-      <x:c r="B15" s="3"/>
-      <x:c r="C15" s="3"/>
-      <x:c r="D15" s="3"/>
-      <x:c r="E15" s="3"/>
-      <x:c r="F15" s="3"/>
-      <x:c r="G15" s="3"/>
-    </x:row>
-    <x:row r="16" ht="24" customHeight="1">
-      <x:c r="A16" s="3"/>
-      <x:c r="B16" s="3"/>
-      <x:c r="C16" s="3"/>
-      <x:c r="D16" s="3"/>
-      <x:c r="E16" s="3"/>
-      <x:c r="F16" s="3"/>
-      <x:c r="G16" s="3"/>
-    </x:row>
-    <x:row r="17" ht="24" customHeight="1">
-      <x:c r="A17" s="3"/>
-      <x:c r="B17" s="3"/>
-      <x:c r="C17" s="3"/>
-      <x:c r="D17" s="3"/>
-      <x:c r="E17" s="3"/>
-      <x:c r="F17" s="3"/>
-      <x:c r="G17" s="3"/>
+    <x:row r="15" ht="135" customHeight="1">
+      <x:c r="A15" s="49" t="str">
+        <x:v>EQ-61</x:v>
+      </x:c>
+      <x:c r="B15" s="51" t="str">
+        <x:v>NVIDIA GeForce RTX 5070, 12 GB GDDR7</x:v>
+      </x:c>
+      <x:c r="C15" s="52" t="n">
+        <x:f>Inventory!D68</x:f>
+        <x:v>799.99</x:v>
+      </x:c>
+      <x:c r="D15" s="52" t="n">
+        <x:f>Inventory!G68</x:f>
+        <x:v>1600</x:v>
+      </x:c>
+      <x:c r="E15" s="51" t="str">
+        <x:v>250 W total graphics power per reference RTX 5070 card; 500 W for two only if both are loaded simultaneously</x:v>
+      </x:c>
+      <x:c r="F15" s="51" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="G15" s="51" t="str">
+        <x:v>Dated comparable-card US retail reference. Acquired and reported September 23, 2026. Exact board makers and purchase prices were not supplied. Best Buy listed a PNY RTX 5070 12 GB card for $799.99 each; two comparable cards are used for this planning estimate. Actual card specifications and availability may differ.
+Price: https://www.bestbuy.com/product/pny-geforce-rtx-5070-12gb-oc-gddr7-pci-express-5-0-graphics-card-with-triple-fan-black/6620352
+Power: NVIDIA RTX 5070 reference total graphics power is 250 W per card, not measured wall draw. Partner boards can differ. Host, dock and power-supply losses are additional; the Lab's single dock cannot run both cards at once.
+https://www.nvidia.com/en-us/geforce/graphics-cards/50-series/rtx-5070-family/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="135" customHeight="1">
+      <x:c r="A16" s="49" t="str">
+        <x:v>EQ-62</x:v>
+      </x:c>
+      <x:c r="B16" s="51" t="str">
+        <x:v>NVIDIA GeForce RTX 4070 SUPER, 12 GB GDDR6X</x:v>
+      </x:c>
+      <x:c r="C16" s="52" t="n">
+        <x:f>Inventory!D69</x:f>
+        <x:v>799</x:v>
+      </x:c>
+      <x:c r="D16" s="52" t="n">
+        <x:f>Inventory!G69</x:f>
+        <x:v>799</x:v>
+      </x:c>
+      <x:c r="E16" s="51" t="str">
+        <x:v>220 W graphics card power for the NVIDIA reference RTX 4070 SUPER</x:v>
+      </x:c>
+      <x:c r="F16" s="51" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="G16" s="51" t="str">
+        <x:v>Dated comparable-card US retail reference. Acquired and reported September 23, 2026. Exact board maker and purchase price were not supplied. Walmart listed a PNY RTX 4070 SUPER 12 GB for $799.00; this is a comparable planning reference.
+Price: https://www.walmart.com/ip/5265483626
+Power: NVIDIA specifies 220 W graphics card power for the reference design, not measured wall draw for this acquired board. Host, dock and power-supply losses are additional; a partner board can differ.
+https://www.nvidia.com/en-au/geforce/graphics-cards/40-series/rtx-4070-family/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="135" customHeight="1">
+      <x:c r="A17" s="49" t="str">
+        <x:v>EQ-63</x:v>
+      </x:c>
+      <x:c r="B17" s="51" t="str">
+        <x:v>Intel Arc Pro B70, 32 GB GDDR6</x:v>
+      </x:c>
+      <x:c r="C17" s="52" t="n">
+        <x:f>Inventory!D70</x:f>
+        <x:v>1299.99</x:v>
+      </x:c>
+      <x:c r="D17" s="52" t="n">
+        <x:f>Inventory!G70</x:f>
+        <x:v>1300</x:v>
+      </x:c>
+      <x:c r="E17" s="51" t="str">
+        <x:v>160-290 W board-power range across Intel Arc Pro B70 designs; Intel-branded card is 230 W</x:v>
+      </x:c>
+      <x:c r="F17" s="51" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="G17" s="51" t="str">
+        <x:v>Dated comparable-card US retail reference. Acquired and reported September 23, 2026 as a B70. This registry assumes Intel Arc Pro B70; the exact board maker and paid price were not supplied. Newegg listed an ASRock Arc Pro B70 CT 32 GB for $1,299.99. The listing is a comparable replacement reference, not an identification of the acquired card.
+Price: https://www.newegg.com/asrock-b70-ct-intel-arc-pro-b70-32gb-graphics-card/p/N82E16814930149
+Power: Intel publishes 160-290 W for B70 designs and 230 W for the Intel-branded card. The acquired board is unconfirmed, so no single wattage is assigned. These are card specifications, not measured Lab wall draw; host and power-supply losses are additional.
+https://www.intel.com/content/dam/www/central-libraries/us/en/documents/2026-03/datasheet-b70-gpu.pdf</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="24" customHeight="1">
       <x:c r="A18" s="3"/>
@@ -4566,10 +4737,37 @@
       <x:c r="F18" s="3"/>
       <x:c r="G18" s="3"/>
     </x:row>
+    <x:row r="19" ht="24" customHeight="1">
+      <x:c r="A19" s="3"/>
+      <x:c r="B19" s="3"/>
+      <x:c r="C19" s="3"/>
+      <x:c r="D19" s="3"/>
+      <x:c r="E19" s="3"/>
+      <x:c r="F19" s="3"/>
+      <x:c r="G19" s="3"/>
+    </x:row>
+    <x:row r="20" ht="24" customHeight="1">
+      <x:c r="A20" s="3"/>
+      <x:c r="B20" s="3"/>
+      <x:c r="C20" s="3"/>
+      <x:c r="D20" s="3"/>
+      <x:c r="E20" s="3"/>
+      <x:c r="F20" s="3"/>
+      <x:c r="G20" s="3"/>
+    </x:row>
+    <x:row r="21" ht="24" customHeight="1">
+      <x:c r="A21" s="3"/>
+      <x:c r="B21" s="3"/>
+      <x:c r="C21" s="3"/>
+      <x:c r="D21" s="3"/>
+      <x:c r="E21" s="3"/>
+      <x:c r="F21" s="3"/>
+      <x:c r="G21" s="3"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf832c33745a94a08"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R802cb683e01c4ca8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Update project status and add TYAN GPU server
</commit_message>
<xml_diff>
--- a/public/lab/hack-lab-inventory.xlsx
+++ b/public/lab/hack-lab-inventory.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R7f7b50554c954ee0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory" sheetId="2" r:id="Ra10e0dd746a14ef2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Power model" sheetId="3" r:id="R7b2434715ba344c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device references" sheetId="4" r:id="Rad036bf103cb4bdb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R05b38e0d95c244a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory" sheetId="2" r:id="R1e3ac9adee0d4107"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Power model" sheetId="3" r:id="R2028cbe5862544a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device references" sheetId="4" r:id="R8b995b02ef8a49e8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -294,8 +294,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="LabInventory" displayName="LabInventory" ref="A7:J70" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A7:J70"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="LabInventory" displayName="LabInventory" ref="A7:J71" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A7:J71"/>
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="Item ID"/>
     <x:tableColumn id="2" name="Equipment and specifications"/>
@@ -329,8 +329,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DeviceReferences" displayName="DeviceReferences" ref="A6:G17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A6:G17"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DeviceReferences" displayName="DeviceReferences" ref="A6:G18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A6:G18"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="Item ID"/>
     <x:tableColumn id="2" name="Equipment"/>
@@ -601,8 +601,8 @@
         <x:v>Compute and add-ons</x:v>
       </x:c>
       <x:c r="B7" s="15" t="n">
-        <x:f>IF(COUNTIFS('Inventory'!J8:J70,A7,'Inventory'!G8:G70,"Missing input")=0,SUMIFS('Inventory'!G8:G70,'Inventory'!J8:J70,A7),"Missing input")</x:f>
-        <x:v>32331</x:v>
+        <x:f>IF(COUNTIFS('Inventory'!J8:J71,A7,'Inventory'!G8:G71,"Missing input")=0,SUMIFS('Inventory'!G8:G71,'Inventory'!J8:J71,A7),"Missing input")</x:f>
+        <x:v>33631</x:v>
       </x:c>
       <x:c r="C7" s="3"/>
       <x:c r="D7" s="3"/>
@@ -612,7 +612,7 @@
         <x:v>Rack and shared</x:v>
       </x:c>
       <x:c r="B8" s="15" t="n">
-        <x:f>IF(COUNTIFS('Inventory'!J8:J70,A8,'Inventory'!G8:G70,"Missing input")=0,SUMIFS('Inventory'!G8:G70,'Inventory'!J8:J70,A8),"Missing input")</x:f>
+        <x:f>IF(COUNTIFS('Inventory'!J8:J71,A8,'Inventory'!G8:G71,"Missing input")=0,SUMIFS('Inventory'!G8:G71,'Inventory'!J8:J71,A8),"Missing input")</x:f>
         <x:v>2613</x:v>
       </x:c>
       <x:c r="C8" s="3"/>
@@ -624,7 +624,7 @@
       </x:c>
       <x:c r="B9" s="19" t="n">
         <x:f>IF(COUNT(B7:B8)=2,SUM(B7:B8),"Missing input")</x:f>
-        <x:v>34944</x:v>
+        <x:v>36244</x:v>
       </x:c>
       <x:c r="C9" s="3"/>
       <x:c r="D9" s="3"/>
@@ -634,8 +634,8 @@
         <x:v>Priced equipment subtotal</x:v>
       </x:c>
       <x:c r="B10" s="15" t="n">
-        <x:f>SUM('Inventory'!G8:G70)</x:f>
-        <x:v>34944</x:v>
+        <x:f>SUM('Inventory'!G8:G71)</x:f>
+        <x:v>36244</x:v>
       </x:c>
       <x:c r="C10" s="3"/>
       <x:c r="D10" s="3"/>
@@ -3392,50 +3392,74 @@
 https://www.newegg.com/asrock-b70-ct-intel-arc-pro-b70-32gb-graphics-card/p/N82E16814930149</x:v>
       </x:c>
     </x:row>
-    <x:row r="71" ht="24" customHeight="1">
-      <x:c r="A71" s="3"/>
-      <x:c r="B71" s="3"/>
-      <x:c r="C71" s="3"/>
-      <x:c r="D71" s="3"/>
-      <x:c r="E71" s="3"/>
-      <x:c r="F71" s="3"/>
-      <x:c r="G71" s="3"/>
-      <x:c r="H71" s="3"/>
-      <x:c r="I71" s="3"/>
-      <x:c r="J71" s="3"/>
+    <x:row r="71" ht="105" customHeight="1">
+      <x:c r="A71" s="16" t="str">
+        <x:v>EQ-64</x:v>
+      </x:c>
+      <x:c r="B71" s="43" t="str">
+        <x:v>TYAN FT77C-B7079 GPU server, 2 × Xeon E5-2660 v3, 128 GB RAM</x:v>
+      </x:c>
+      <x:c r="C71" s="38" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D71" s="39" t="n">
+        <x:v>1299.88</x:v>
+      </x:c>
+      <x:c r="E71" s="39" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F71" s="40" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G71" s="41" t="n">
+        <x:f>IF(COUNT(C71:F71)=4,ROUND(C71*(D71+E71),0)+F71,"Missing input")</x:f>
+        <x:v>1300</x:v>
+      </x:c>
+      <x:c r="H71" s="42" t="str">
+        <x:v>none</x:v>
+      </x:c>
+      <x:c r="I71" s="30" t="str">
+        <x:v>Acquired 4U server; installation, GPU population, input voltage, and measured wall draw unconfirmed. Excluded from configured-lab power totals</x:v>
+      </x:c>
+      <x:c r="J71" s="30" t="str">
+        <x:v>Compute and add-ons</x:v>
+      </x:c>
       <x:c r="K71" s="3"/>
-      <x:c r="L71" s="3"/>
-    </x:row>
-    <x:row r="72" ht="30" customHeight="1">
-      <x:c r="A72" s="18" t="str">
-        <x:v>Total equipment cost estimate</x:v>
-      </x:c>
-      <x:c r="B72" s="18"/>
-      <x:c r="C72" s="18"/>
-      <x:c r="D72" s="18"/>
-      <x:c r="E72" s="18"/>
-      <x:c r="F72" s="18"/>
-      <x:c r="G72" s="19" t="n">
-        <x:f>IF(COUNT(G8:G70)=ROWS(G8:G70),SUM(G8:G70),"Missing input")</x:f>
-        <x:v>34944</x:v>
-      </x:c>
-      <x:c r="H72" s="18"/>
-      <x:c r="I72" s="18"/>
-      <x:c r="J72" s="18"/>
+      <x:c r="L71" s="32" t="str">
+        <x:v>Acquired and reported September 23, 2026. Purchase price was not supplied. An eBay listing with the stated TYAN FT77CB7079, dual E5-2660 v3, and 128 GB RAM configuration displayed $1,299.88 with free domestic shipping when checked September 23. The listing's item-specific motherboard identifiers appear inconsistent with its title, so this is a provisional market reference rather than confirmation of the acquired unit or amount paid.
+https://www.ebay.com/itm/188585858524</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72" ht="24" customHeight="1">
+      <x:c r="A72" s="3"/>
+      <x:c r="B72" s="3"/>
+      <x:c r="C72" s="3"/>
+      <x:c r="D72" s="3"/>
+      <x:c r="E72" s="3"/>
+      <x:c r="F72" s="3"/>
+      <x:c r="G72" s="3"/>
+      <x:c r="H72" s="3"/>
+      <x:c r="I72" s="3"/>
+      <x:c r="J72" s="3"/>
       <x:c r="K72" s="3"/>
       <x:c r="L72" s="3"/>
     </x:row>
-    <x:row r="73" ht="24" customHeight="1">
-      <x:c r="A73" s="3"/>
-      <x:c r="B73" s="3"/>
-      <x:c r="C73" s="3"/>
-      <x:c r="D73" s="3"/>
-      <x:c r="E73" s="3"/>
-      <x:c r="F73" s="3"/>
-      <x:c r="G73" s="3"/>
-      <x:c r="H73" s="3"/>
-      <x:c r="I73" s="3"/>
-      <x:c r="J73" s="3"/>
+    <x:row r="73" ht="30" customHeight="1">
+      <x:c r="A73" s="18" t="str">
+        <x:v>Total equipment cost estimate</x:v>
+      </x:c>
+      <x:c r="B73" s="18"/>
+      <x:c r="C73" s="18"/>
+      <x:c r="D73" s="18"/>
+      <x:c r="E73" s="18"/>
+      <x:c r="F73" s="18"/>
+      <x:c r="G73" s="19" t="n">
+        <x:f>IF(COUNT(G8:G71)=ROWS(G8:G71),SUM(G8:G71),"Missing input")</x:f>
+        <x:v>36244</x:v>
+      </x:c>
+      <x:c r="H73" s="18"/>
+      <x:c r="I73" s="18"/>
+      <x:c r="J73" s="18"/>
       <x:c r="K73" s="3"/>
       <x:c r="L73" s="3"/>
     </x:row>
@@ -3467,21 +3491,35 @@
       <x:c r="K75" s="3"/>
       <x:c r="L75" s="3"/>
     </x:row>
+    <x:row r="76" ht="24" customHeight="1">
+      <x:c r="A76" s="3"/>
+      <x:c r="B76" s="3"/>
+      <x:c r="C76" s="3"/>
+      <x:c r="D76" s="3"/>
+      <x:c r="E76" s="3"/>
+      <x:c r="F76" s="3"/>
+      <x:c r="G76" s="3"/>
+      <x:c r="H76" s="3"/>
+      <x:c r="I76" s="3"/>
+      <x:c r="J76" s="3"/>
+      <x:c r="K76" s="3"/>
+      <x:c r="L76" s="3"/>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="G8:G70">
+  <x:conditionalFormatting sqref="G8:G71">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Missing input"/>
   </x:conditionalFormatting>
   <x:dataValidations count="2">
-    <x:dataValidation type="whole" operator="greaterThanOrEqual" sqref="C8:C70">
+    <x:dataValidation type="whole" operator="greaterThanOrEqual" sqref="C8:C71">
       <x:formula1>0</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="decimal" operator="greaterThanOrEqual" sqref="D8:E70">
+    <x:dataValidation type="decimal" operator="greaterThanOrEqual" sqref="D8:E71">
       <x:formula1>0</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26e774bc00c84f92"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re028e8060a894031"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4325,7 +4363,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R60913cfa222a4280"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b8ef094af854bf8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4728,14 +4766,33 @@
 https://www.intel.com/content/dam/www/central-libraries/us/en/documents/2026-03/datasheet-b70-gpu.pdf</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="24" customHeight="1">
-      <x:c r="A18" s="3"/>
-      <x:c r="B18" s="3"/>
-      <x:c r="C18" s="3"/>
-      <x:c r="D18" s="3"/>
-      <x:c r="E18" s="3"/>
-      <x:c r="F18" s="3"/>
-      <x:c r="G18" s="3"/>
+    <x:row r="18" ht="135" customHeight="1">
+      <x:c r="A18" s="49" t="str">
+        <x:v>EQ-64</x:v>
+      </x:c>
+      <x:c r="B18" s="51" t="str">
+        <x:v>TYAN FT77C-B7079 GPU server, 2 × Xeon E5-2660 v3, 128 GB RAM</x:v>
+      </x:c>
+      <x:c r="C18" s="52" t="n">
+        <x:f>Inventory!D71</x:f>
+        <x:v>1299.88</x:v>
+      </x:c>
+      <x:c r="D18" s="52" t="n">
+        <x:f>Inventory!G71</x:f>
+        <x:v>1300</x:v>
+      </x:c>
+      <x:c r="E18" s="51" t="str">
+        <x:v>Two CPUs rated 105 W TDP each. Chassis PSU output capacity: 2,000 W on 100-127 V AC or 3,200 W on 200-240 V AC; actual wall draw is unknown</x:v>
+      </x:c>
+      <x:c r="F18" s="51" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="G18" s="51" t="str">
+        <x:v>Dated comparable used-server US retail reference. Acquired and reported September 23, 2026. Purchase price was not supplied. An eBay listing with the stated TYAN FT77CB7079, dual E5-2660 v3, and 128 GB RAM configuration displayed $1,299.88 with free domestic shipping when checked September 23. The listing's item-specific motherboard identifiers appear inconsistent with its title, so this is a provisional market reference rather than confirmation of the acquired unit or amount paid.
+Price: https://www.ebay.com/itm/188585858524
+Power: Intel specifies 105 W TDP per E5-2660 v3. TYAN specifies 2,000 W or 3,200 W power-supply output capacity depending on input voltage. CPU TDP is not measured electrical consumption, and PSU capacity is not server draw. Fans, memory, storage, GPU selection, utilization, and PSU losses determine actual wall power. Meter the installed system before revising Lab or hosting power estimates.
+https://www.intel.com/content/www/us/en/ark/products/series/78583/intel-xeon-processor-e5-v3-family.html | https://ftp1.tyan.com/pub/doc/FT77C-B7079_UG_V1.0q.pdf</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="24" customHeight="1">
       <x:c r="A19" s="3"/>
@@ -4764,10 +4821,19 @@
       <x:c r="F21" s="3"/>
       <x:c r="G21" s="3"/>
     </x:row>
+    <x:row r="22" ht="24" customHeight="1">
+      <x:c r="A22" s="3"/>
+      <x:c r="B22" s="3"/>
+      <x:c r="C22" s="3"/>
+      <x:c r="D22" s="3"/>
+      <x:c r="E22" s="3"/>
+      <x:c r="F22" s="3"/>
+      <x:c r="G22" s="3"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R802cb683e01c4ca8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R197830300f78472b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add Dell R730 and Omada switch to lab inventory
</commit_message>
<xml_diff>
--- a/public/lab/hack-lab-inventory.xlsx
+++ b/public/lab/hack-lab-inventory.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R05b38e0d95c244a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory" sheetId="2" r:id="R1e3ac9adee0d4107"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Power model" sheetId="3" r:id="R2028cbe5862544a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device references" sheetId="4" r:id="R8b995b02ef8a49e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rbece1df28aea49e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory" sheetId="2" r:id="R21be04b36db84dbc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Power model" sheetId="3" r:id="R706818d1d587497b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device references" sheetId="4" r:id="Rfc4737771fd94477"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -294,8 +294,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="LabInventory" displayName="LabInventory" ref="A7:J71" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A7:J71"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="LabInventory" displayName="LabInventory" ref="A7:J73" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A7:J73"/>
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="Item ID"/>
     <x:tableColumn id="2" name="Equipment and specifications"/>
@@ -329,8 +329,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DeviceReferences" displayName="DeviceReferences" ref="A6:G18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A6:G18"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DeviceReferences" displayName="DeviceReferences" ref="A6:G20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A6:G20"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="Item ID"/>
     <x:tableColumn id="2" name="Equipment"/>
@@ -575,7 +575,7 @@
         <x:v>Snapshot</x:v>
       </x:c>
       <x:c r="B4" s="6" t="n">
-        <x:v>46288.5</x:v>
+        <x:v>46293.5</x:v>
       </x:c>
       <x:c r="C4" s="3"/>
       <x:c r="D4" s="3"/>
@@ -601,8 +601,8 @@
         <x:v>Compute and add-ons</x:v>
       </x:c>
       <x:c r="B7" s="15" t="n">
-        <x:f>IF(COUNTIFS('Inventory'!J8:J71,A7,'Inventory'!G8:G71,"Missing input")=0,SUMIFS('Inventory'!G8:G71,'Inventory'!J8:J71,A7),"Missing input")</x:f>
-        <x:v>33631</x:v>
+        <x:f>IF(COUNTIFS('Inventory'!J8:J73,A7,'Inventory'!G8:G73,"Missing input")=0,SUMIFS('Inventory'!G8:G73,'Inventory'!J8:J73,A7),"Missing input")</x:f>
+        <x:v>36482</x:v>
       </x:c>
       <x:c r="C7" s="3"/>
       <x:c r="D7" s="3"/>
@@ -612,8 +612,8 @@
         <x:v>Rack and shared</x:v>
       </x:c>
       <x:c r="B8" s="15" t="n">
-        <x:f>IF(COUNTIFS('Inventory'!J8:J71,A8,'Inventory'!G8:G71,"Missing input")=0,SUMIFS('Inventory'!G8:G71,'Inventory'!J8:J71,A8),"Missing input")</x:f>
-        <x:v>2613</x:v>
+        <x:f>IF(COUNTIFS('Inventory'!J8:J73,A8,'Inventory'!G8:G73,"Missing input")=0,SUMIFS('Inventory'!G8:G73,'Inventory'!J8:J73,A8),"Missing input")</x:f>
+        <x:v>2853</x:v>
       </x:c>
       <x:c r="C8" s="3"/>
       <x:c r="D8" s="3"/>
@@ -624,7 +624,7 @@
       </x:c>
       <x:c r="B9" s="19" t="n">
         <x:f>IF(COUNT(B7:B8)=2,SUM(B7:B8),"Missing input")</x:f>
-        <x:v>36244</x:v>
+        <x:v>39335</x:v>
       </x:c>
       <x:c r="C9" s="3"/>
       <x:c r="D9" s="3"/>
@@ -634,8 +634,8 @@
         <x:v>Priced equipment subtotal</x:v>
       </x:c>
       <x:c r="B10" s="15" t="n">
-        <x:f>SUM('Inventory'!G8:G71)</x:f>
-        <x:v>36244</x:v>
+        <x:f>SUM('Inventory'!G8:G73)</x:f>
+        <x:v>39335</x:v>
       </x:c>
       <x:c r="C10" s="3"/>
       <x:c r="D10" s="3"/>
@@ -826,7 +826,7 @@
     </x:row>
     <x:row r="32" ht="24" customHeight="1">
       <x:c r="A32" s="20" t="str">
-        <x:v>Original references: September 11–12, 2026; added devices researched through September 23.</x:v>
+        <x:v>Original references: September 11–12, 2026; added devices researched through September 28.</x:v>
       </x:c>
       <x:c r="B32" s="3"/>
       <x:c r="C32" s="3"/>
@@ -3430,38 +3430,81 @@
 https://www.ebay.com/itm/188585858524</x:v>
       </x:c>
     </x:row>
-    <x:row r="72" ht="24" customHeight="1">
-      <x:c r="A72" s="3"/>
-      <x:c r="B72" s="3"/>
-      <x:c r="C72" s="3"/>
-      <x:c r="D72" s="3"/>
-      <x:c r="E72" s="3"/>
-      <x:c r="F72" s="3"/>
-      <x:c r="G72" s="3"/>
-      <x:c r="H72" s="3"/>
-      <x:c r="I72" s="3"/>
-      <x:c r="J72" s="3"/>
+    <x:row r="72" ht="77" customHeight="1">
+      <x:c r="A72" s="3" t="str">
+        <x:v>EQ-65</x:v>
+      </x:c>
+      <x:c r="B72" s="30" t="str">
+        <x:v>Dell PowerEdge R730, 16-bay SFF, 2.50 GHz 24-core, 512 GB RAM, 16 caddies</x:v>
+      </x:c>
+      <x:c r="C72" s="38" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D72" s="39" t="n">
+        <x:v>2850.95</x:v>
+      </x:c>
+      <x:c r="E72" s="39" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F72" s="40" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G72" s="41" t="n">
+        <x:f>IF(COUNT(C72:F72)=4,ROUND(C72*(D72+E72),0)+F72,"Missing input")</x:f>
+        <x:v>2851</x:v>
+      </x:c>
+      <x:c r="H72" s="42" t="str">
+        <x:v>none</x:v>
+      </x:c>
+      <x:c r="I72" s="30" t="str">
+        <x:v>Acquired server; CPU/PSU variants, drives, installation, and measured wall draw unconfirmed. Excluded from configured-lab power totals</x:v>
+      </x:c>
+      <x:c r="J72" s="30" t="str">
+        <x:v>Compute and add-ons</x:v>
+      </x:c>
       <x:c r="K72" s="3"/>
-      <x:c r="L72" s="3"/>
-    </x:row>
-    <x:row r="73" ht="30" customHeight="1">
-      <x:c r="A73" s="18" t="str">
-        <x:v>Total equipment cost estimate</x:v>
-      </x:c>
-      <x:c r="B73" s="18"/>
-      <x:c r="C73" s="18"/>
-      <x:c r="D73" s="18"/>
-      <x:c r="E73" s="18"/>
-      <x:c r="F73" s="18"/>
-      <x:c r="G73" s="19" t="n">
-        <x:f>IF(COUNT(G8:G71)=ROWS(G8:G71),SUM(G8:G71),"Missing input")</x:f>
-        <x:v>36244</x:v>
-      </x:c>
-      <x:c r="H73" s="18"/>
-      <x:c r="I73" s="18"/>
-      <x:c r="J73" s="18"/>
+      <x:c r="L72" s="32" t="str">
+        <x:v>Acquired and reported September 28, 2026. Owner purchase price and exact CPU/PSU models were not supplied. TechMikeNY's matching 16-bay, 2.50 GHz 24-core, 512 GB, 16-caddie R730 listing showed $2,850.95 on September 28. This is a comparable market reference, not the amount paid. Caddies do not imply drives are installed.
+https://www.ebay.com/str/techmikeny/Dell-PowerEdge-R730/_i.html?store_cat=15884377015</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73" ht="77" customHeight="1">
+      <x:c r="A73" s="16" t="str">
+        <x:v>EQ-66</x:v>
+      </x:c>
+      <x:c r="B73" s="43" t="str">
+        <x:v>Omada 10G network switch, exact model unconfirmed</x:v>
+      </x:c>
+      <x:c r="C73" s="38" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D73" s="39" t="n">
+        <x:v>239.99</x:v>
+      </x:c>
+      <x:c r="E73" s="39" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F73" s="40" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G73" s="41" t="n">
+        <x:f>IF(COUNT(C73:F73)=4,ROUND(C73*(D73+E73),0)+F73,"Missing input")</x:f>
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="H73" s="42" t="str">
+        <x:v>none</x:v>
+      </x:c>
+      <x:c r="I73" s="30" t="str">
+        <x:v>Acquired network switch; exact model, installation, and whether it augments or replaces the existing switch are unconfirmed. Excluded from configured-lab power totals</x:v>
+      </x:c>
+      <x:c r="J73" s="30" t="str">
+        <x:v>Rack and shared</x:v>
+      </x:c>
       <x:c r="K73" s="3"/>
-      <x:c r="L73" s="3"/>
+      <x:c r="L73" s="32" t="str">
+        <x:v>Acquired and reported September 28, 2026. Exact Omada model and paid price were not supplied. B&amp;H listed the eight-port 10G SFP+ SX3008F for $239.99 on September 28. This is a provisional comparable price, not identification of the acquired switch.
+https://www.bhphotovideo.com/c/product/1684305-REG/tp_link_tl_sx3008f_jetstream_8_port_10ge.html</x:v>
+      </x:c>
     </x:row>
     <x:row r="74" ht="24" customHeight="1">
       <x:c r="A74" s="3"/>
@@ -3477,17 +3520,22 @@
       <x:c r="K74" s="3"/>
       <x:c r="L74" s="3"/>
     </x:row>
-    <x:row r="75" ht="24" customHeight="1">
-      <x:c r="A75" s="3"/>
-      <x:c r="B75" s="3"/>
-      <x:c r="C75" s="3"/>
-      <x:c r="D75" s="3"/>
-      <x:c r="E75" s="3"/>
-      <x:c r="F75" s="3"/>
-      <x:c r="G75" s="3"/>
-      <x:c r="H75" s="3"/>
-      <x:c r="I75" s="3"/>
-      <x:c r="J75" s="3"/>
+    <x:row r="75" ht="30" customHeight="1">
+      <x:c r="A75" s="18" t="str">
+        <x:v>Total equipment cost estimate</x:v>
+      </x:c>
+      <x:c r="B75" s="18"/>
+      <x:c r="C75" s="18"/>
+      <x:c r="D75" s="18"/>
+      <x:c r="E75" s="18"/>
+      <x:c r="F75" s="18"/>
+      <x:c r="G75" s="19" t="n">
+        <x:f>IF(COUNT(G8:G73)=ROWS(G8:G73),SUM(G8:G73),"Missing input")</x:f>
+        <x:v>39335</x:v>
+      </x:c>
+      <x:c r="H75" s="18"/>
+      <x:c r="I75" s="18"/>
+      <x:c r="J75" s="18"/>
       <x:c r="K75" s="3"/>
       <x:c r="L75" s="3"/>
     </x:row>
@@ -3505,21 +3553,49 @@
       <x:c r="K76" s="3"/>
       <x:c r="L76" s="3"/>
     </x:row>
+    <x:row r="77" ht="24" customHeight="1">
+      <x:c r="A77" s="3"/>
+      <x:c r="B77" s="3"/>
+      <x:c r="C77" s="3"/>
+      <x:c r="D77" s="3"/>
+      <x:c r="E77" s="3"/>
+      <x:c r="F77" s="3"/>
+      <x:c r="G77" s="3"/>
+      <x:c r="H77" s="3"/>
+      <x:c r="I77" s="3"/>
+      <x:c r="J77" s="3"/>
+      <x:c r="K77" s="3"/>
+      <x:c r="L77" s="3"/>
+    </x:row>
+    <x:row r="78" ht="24" customHeight="1">
+      <x:c r="A78" s="3"/>
+      <x:c r="B78" s="3"/>
+      <x:c r="C78" s="3"/>
+      <x:c r="D78" s="3"/>
+      <x:c r="E78" s="3"/>
+      <x:c r="F78" s="3"/>
+      <x:c r="G78" s="3"/>
+      <x:c r="H78" s="3"/>
+      <x:c r="I78" s="3"/>
+      <x:c r="J78" s="3"/>
+      <x:c r="K78" s="3"/>
+      <x:c r="L78" s="3"/>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="G8:G71">
+  <x:conditionalFormatting sqref="G8:G73">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Missing input"/>
   </x:conditionalFormatting>
   <x:dataValidations count="2">
-    <x:dataValidation type="whole" operator="greaterThanOrEqual" sqref="C8:C71">
+    <x:dataValidation type="whole" operator="greaterThanOrEqual" sqref="C8:C73">
       <x:formula1>0</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="decimal" operator="greaterThanOrEqual" sqref="D8:E71">
+    <x:dataValidation type="decimal" operator="greaterThanOrEqual" sqref="D8:E73">
       <x:formula1>0</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re028e8060a894031"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ab3dc38ded14e76"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4363,7 +4439,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b8ef094af854bf8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c445d9cb06747f3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4794,23 +4870,61 @@
 https://www.intel.com/content/www/us/en/ark/products/series/78583/intel-xeon-processor-e5-v3-family.html | https://ftp1.tyan.com/pub/doc/FT77C-B7079_UG_V1.0q.pdf</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="24" customHeight="1">
-      <x:c r="A19" s="3"/>
-      <x:c r="B19" s="3"/>
-      <x:c r="C19" s="3"/>
-      <x:c r="D19" s="3"/>
-      <x:c r="E19" s="3"/>
-      <x:c r="F19" s="3"/>
-      <x:c r="G19" s="3"/>
-    </x:row>
-    <x:row r="20" ht="24" customHeight="1">
-      <x:c r="A20" s="3"/>
-      <x:c r="B20" s="3"/>
-      <x:c r="C20" s="3"/>
-      <x:c r="D20" s="3"/>
-      <x:c r="E20" s="3"/>
-      <x:c r="F20" s="3"/>
-      <x:c r="G20" s="3"/>
+    <x:row r="19" ht="135" customHeight="1">
+      <x:c r="A19" s="49" t="str">
+        <x:v>EQ-65</x:v>
+      </x:c>
+      <x:c r="B19" s="51" t="str">
+        <x:v>Dell PowerEdge R730, 16-bay SFF, 2.50 GHz 24-core, 512 GB RAM, 16 caddies</x:v>
+      </x:c>
+      <x:c r="C19" s="52" t="n">
+        <x:f>Inventory!D72</x:f>
+        <x:v>2850.95</x:v>
+      </x:c>
+      <x:c r="D19" s="52" t="n">
+        <x:f>Inventory!G72</x:f>
+        <x:v>2851</x:v>
+      </x:c>
+      <x:c r="E19" s="51" t="str">
+        <x:v>Dell R730 supports 495 W, 750 W, or 1,100 W AC PSU options; actual wall draw is unknown</x:v>
+      </x:c>
+      <x:c r="F19" s="51" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="G19" s="51" t="str">
+        <x:v>Dated comparable refurbished-server US retail reference. Acquired and reported September 28, 2026. Owner purchase price and exact CPU/PSU models were not supplied. TechMikeNY's matching 16-bay, 2.50 GHz 24-core, 512 GB, 16-caddie R730 listing showed $2,850.95 on September 28. This is a comparable market reference, not the amount paid. Caddies do not imply drives are installed.
+Price: https://www.ebay.com/str/techmikeny/Dell-PowerEdge-R730/_i.html?store_cat=15884377015
+Power: Dell's published PSU figures are output-capacity options, not consumption. The reported 2.50 GHz / 24-core description does not confirm CPU model or its thermal rating. RAM, storage, load, and PSU losses affect actual draw. Measure the installed server before adding it to the Lab power scenarios.
+https://i.dell.com/sites/doccontent/shared-content/data-sheets/en/documents/dell-poweredge-r730-spec-sheet.pdf</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="135" customHeight="1">
+      <x:c r="A20" s="49" t="str">
+        <x:v>EQ-66</x:v>
+      </x:c>
+      <x:c r="B20" s="51" t="str">
+        <x:v>Omada 10G network switch, exact model unconfirmed</x:v>
+      </x:c>
+      <x:c r="C20" s="52" t="n">
+        <x:f>Inventory!D73</x:f>
+        <x:v>239.99</x:v>
+      </x:c>
+      <x:c r="D20" s="52" t="n">
+        <x:f>Inventory!G73</x:f>
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="E20" s="51" t="str">
+        <x:v>Comparable Omada SX3008F is rated up to 15.46 W; acquired switch model and wall draw unknown</x:v>
+      </x:c>
+      <x:c r="F20" s="51" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="G20" s="51" t="str">
+        <x:v>Dated comparable-switch US retail allowance. Acquired and reported September 28, 2026. Exact Omada model and paid price were not supplied. B&amp;H listed the eight-port 10G SFP+ SX3008F for $239.99 on September 28. This is a provisional comparable price, not identification of the acquired switch.
+Price: https://www.bhphotovideo.com/c/product/1684305-REG/tp_link_tl_sx3008f_jetstream_8_port_10ge.html
+Power: Omada publishes a 15.46 W maximum for the SX3008F v1.20 at 220 V / 50 Hz. The acquired switch could have different ports, PoE capability, and power requirements. Confirm its model and measure or model the installed network before updating Lab scenarios.
+https://www.omadanetworks.com/us/business-networking/omada-switch-aggregation/sx3008f/v1.20/</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="24" customHeight="1">
       <x:c r="A21" s="3"/>
@@ -4830,10 +4944,28 @@
       <x:c r="F22" s="3"/>
       <x:c r="G22" s="3"/>
     </x:row>
+    <x:row r="23" ht="24" customHeight="1">
+      <x:c r="A23" s="3"/>
+      <x:c r="B23" s="3"/>
+      <x:c r="C23" s="3"/>
+      <x:c r="D23" s="3"/>
+      <x:c r="E23" s="3"/>
+      <x:c r="F23" s="3"/>
+      <x:c r="G23" s="3"/>
+    </x:row>
+    <x:row r="24" ht="24" customHeight="1">
+      <x:c r="A24" s="3"/>
+      <x:c r="B24" s="3"/>
+      <x:c r="C24" s="3"/>
+      <x:c r="D24" s="3"/>
+      <x:c r="E24" s="3"/>
+      <x:c r="F24" s="3"/>
+      <x:c r="G24" s="3"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R197830300f78472b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4cf02fa291c54f69"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>